<commit_message>
Update CPU IDD for j, jr, jal
</commit_message>
<xml_diff>
--- a/document/IDD.xlsx
+++ b/document/IDD.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\Document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47090BE-DFE7-4CE4-9182-D31A5AA789FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4AEC23-592B-415F-B0A4-115DBD096B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17235" yWindow="0" windowWidth="11670" windowHeight="15585" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
+    <workbookView xWindow="9885" yWindow="1335" windowWidth="21600" windowHeight="11385" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="410">
   <si>
     <t>top_cpu</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -818,10 +818,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PC ADDR + 4 (ID)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>PC ADDR + 4 (EX)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1230,10 +1226,6 @@
   </si>
   <si>
     <t>w_ex_regwrite</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>w_wb_regwrite</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1648,6 +1640,78 @@
     <t>u_pc_mux
 u_if_id_bridge
 u_id_ex_bridge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_control_unit
+u_id_ex_bridge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_jump_mux
+u_alu_forward_a_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_mem_jump</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_wb_ctr_jump</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jump Flag (MEM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jump Flag (WB)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_wb_regdst_jal_mux_reg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_regdst_jal_mux
+u_wdata_forwarding_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_regdst_jal_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>rt or rd or $ra Register (WB)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_mem_pc_addr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_wb_pc_addr</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_wb_ctr_regwrite</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_regdst_jal_mux
+u_memtoreg_mux</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PC ADDR (ID)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PC ADDR (MEM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PC ADDR (WB)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2631,13 +2695,55 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2649,28 +2755,10 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2680,30 +2768,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3066,31 +3130,31 @@
   <sheetData>
     <row r="1" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="133" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="134"/>
-      <c r="D2" s="134"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="134"/>
-      <c r="G2" s="135"/>
-      <c r="I2" s="119" t="s">
+      <c r="B2" s="141" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="143"/>
+      <c r="I2" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J2" s="121"/>
-      <c r="K2" s="119" t="s">
+      <c r="K2" s="120" t="s">
         <v>96</v>
       </c>
-      <c r="L2" s="120"/>
+      <c r="L2" s="122"/>
       <c r="M2" s="121"/>
-      <c r="O2" s="119" t="s">
+      <c r="O2" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P2" s="121"/>
-      <c r="Q2" s="119" t="s">
+      <c r="Q2" s="120" t="s">
         <v>149</v>
       </c>
-      <c r="R2" s="120"/>
+      <c r="R2" s="122"/>
       <c r="S2" s="121"/>
     </row>
     <row r="3" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3112,24 +3176,24 @@
       <c r="G3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="128" t="s">
+      <c r="I3" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="129"/>
-      <c r="K3" s="130" t="s">
+      <c r="J3" s="131"/>
+      <c r="K3" s="132" t="s">
         <v>109</v>
       </c>
-      <c r="L3" s="131"/>
-      <c r="M3" s="132"/>
-      <c r="O3" s="128" t="s">
+      <c r="L3" s="133"/>
+      <c r="M3" s="134"/>
+      <c r="O3" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="129"/>
-      <c r="Q3" s="130" t="s">
-        <v>233</v>
-      </c>
-      <c r="R3" s="131"/>
-      <c r="S3" s="132"/>
+      <c r="P3" s="131"/>
+      <c r="Q3" s="132" t="s">
+        <v>232</v>
+      </c>
+      <c r="R3" s="133"/>
+      <c r="S3" s="134"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B4" s="35">
@@ -3150,24 +3214,24 @@
       <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="128" t="s">
+      <c r="I4" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J4" s="129"/>
-      <c r="K4" s="128" t="s">
+      <c r="J4" s="131"/>
+      <c r="K4" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="142"/>
-      <c r="M4" s="129"/>
-      <c r="O4" s="128" t="s">
+      <c r="L4" s="135"/>
+      <c r="M4" s="131"/>
+      <c r="O4" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P4" s="129"/>
-      <c r="Q4" s="128" t="s">
+      <c r="P4" s="131"/>
+      <c r="Q4" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R4" s="142"/>
-      <c r="S4" s="129"/>
+      <c r="R4" s="135"/>
+      <c r="S4" s="131"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="54">
@@ -3188,24 +3252,24 @@
       <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="122" t="s">
+      <c r="I5" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="123"/>
-      <c r="K5" s="124" t="s">
+      <c r="J5" s="137"/>
+      <c r="K5" s="138" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="125"/>
-      <c r="M5" s="126"/>
-      <c r="O5" s="122" t="s">
+      <c r="L5" s="119"/>
+      <c r="M5" s="139"/>
+      <c r="O5" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="123"/>
-      <c r="Q5" s="124" t="s">
+      <c r="P5" s="137"/>
+      <c r="Q5" s="138" t="s">
         <v>150</v>
       </c>
-      <c r="R5" s="125"/>
-      <c r="S5" s="126"/>
+      <c r="R5" s="119"/>
+      <c r="S5" s="139"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="55">
@@ -3229,22 +3293,22 @@
       <c r="I6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="127" t="s">
+      <c r="J6" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K6" s="127"/>
-      <c r="L6" s="127"/>
+      <c r="K6" s="128"/>
+      <c r="L6" s="128"/>
       <c r="M6" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="127" t="s">
+      <c r="P6" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q6" s="127"/>
-      <c r="R6" s="127"/>
+      <c r="Q6" s="128"/>
+      <c r="R6" s="128"/>
       <c r="S6" s="69" t="s">
         <v>8</v>
       </c>
@@ -3271,22 +3335,22 @@
       <c r="I7" s="70">
         <v>1</v>
       </c>
-      <c r="J7" s="136" t="s">
+      <c r="J7" s="140" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="136"/>
-      <c r="L7" s="136"/>
+      <c r="K7" s="140"/>
+      <c r="L7" s="140"/>
       <c r="M7" s="71" t="s">
         <v>132</v>
       </c>
       <c r="O7" s="87">
         <v>1</v>
       </c>
-      <c r="P7" s="143" t="s">
+      <c r="P7" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="143"/>
-      <c r="R7" s="143"/>
+      <c r="Q7" s="129"/>
+      <c r="R7" s="129"/>
       <c r="S7" s="88" t="s">
         <v>132</v>
       </c>
@@ -3328,11 +3392,11 @@
       <c r="O8" s="80">
         <v>2</v>
       </c>
-      <c r="P8" s="125" t="s">
+      <c r="P8" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="125"/>
-      <c r="R8" s="125"/>
+      <c r="Q8" s="119"/>
+      <c r="R8" s="119"/>
       <c r="S8" s="82" t="s">
         <v>133</v>
       </c>
@@ -3506,15 +3570,15 @@
       <c r="G12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="137" t="s">
+      <c r="I12" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="138"/>
-      <c r="K12" s="139" t="s">
+      <c r="J12" s="124"/>
+      <c r="K12" s="125" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="140"/>
-      <c r="M12" s="141"/>
+      <c r="L12" s="126"/>
+      <c r="M12" s="127"/>
       <c r="O12" s="72">
         <v>3</v>
       </c>
@@ -3637,15 +3701,15 @@
       </c>
     </row>
     <row r="16" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O16" s="137" t="s">
+      <c r="O16" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P16" s="138"/>
-      <c r="Q16" s="139" t="s">
-        <v>236</v>
-      </c>
-      <c r="R16" s="140"/>
-      <c r="S16" s="141"/>
+      <c r="P16" s="124"/>
+      <c r="Q16" s="125" t="s">
+        <v>235</v>
+      </c>
+      <c r="R16" s="126"/>
+      <c r="S16" s="127"/>
     </row>
     <row r="17" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="90" t="s">
@@ -3673,7 +3737,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D18" s="1">
         <v>1</v>
@@ -3687,23 +3751,23 @@
       <c r="G18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="I18" s="119" t="s">
+      <c r="I18" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J18" s="121"/>
-      <c r="K18" s="119" t="s">
+      <c r="K18" s="120" t="s">
         <v>103</v>
       </c>
-      <c r="L18" s="120"/>
+      <c r="L18" s="122"/>
       <c r="M18" s="121"/>
-      <c r="O18" s="119" t="s">
+      <c r="O18" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P18" s="121"/>
-      <c r="Q18" s="119" t="s">
+      <c r="Q18" s="120" t="s">
         <v>159</v>
       </c>
-      <c r="R18" s="120"/>
+      <c r="R18" s="122"/>
       <c r="S18" s="121"/>
     </row>
     <row r="19" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -3712,7 +3776,7 @@
         <v>2</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D19" s="1">
         <v>4</v>
@@ -3726,24 +3790,24 @@
       <c r="G19" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="I19" s="128" t="s">
+      <c r="I19" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J19" s="129"/>
-      <c r="K19" s="130" t="s">
+      <c r="J19" s="131"/>
+      <c r="K19" s="132" t="s">
         <v>110</v>
       </c>
-      <c r="L19" s="131"/>
-      <c r="M19" s="132"/>
-      <c r="O19" s="128" t="s">
+      <c r="L19" s="133"/>
+      <c r="M19" s="134"/>
+      <c r="O19" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P19" s="129"/>
-      <c r="Q19" s="130" t="s">
-        <v>233</v>
-      </c>
-      <c r="R19" s="131"/>
-      <c r="S19" s="132"/>
+      <c r="P19" s="131"/>
+      <c r="Q19" s="132" t="s">
+        <v>232</v>
+      </c>
+      <c r="R19" s="133"/>
+      <c r="S19" s="134"/>
     </row>
     <row r="20" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B20" s="33">
@@ -3751,38 +3815,38 @@
         <v>3</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D20" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F20" s="103" t="s">
         <v>75</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="I20" s="128" t="s">
+        <v>353</v>
+      </c>
+      <c r="I20" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J20" s="129"/>
-      <c r="K20" s="130" t="s">
+      <c r="J20" s="131"/>
+      <c r="K20" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="L20" s="131"/>
-      <c r="M20" s="132"/>
-      <c r="O20" s="128" t="s">
+      <c r="L20" s="133"/>
+      <c r="M20" s="134"/>
+      <c r="O20" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P20" s="129"/>
-      <c r="Q20" s="128" t="s">
+      <c r="P20" s="131"/>
+      <c r="Q20" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R20" s="142"/>
-      <c r="S20" s="129"/>
+      <c r="R20" s="135"/>
+      <c r="S20" s="131"/>
     </row>
     <row r="21" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="33">
@@ -3790,38 +3854,38 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D21" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F21" s="103" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="I21" s="122" t="s">
+        <v>355</v>
+      </c>
+      <c r="I21" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J21" s="123"/>
-      <c r="K21" s="124" t="s">
+      <c r="J21" s="137"/>
+      <c r="K21" s="138" t="s">
         <v>124</v>
       </c>
-      <c r="L21" s="125"/>
-      <c r="M21" s="126"/>
-      <c r="O21" s="122" t="s">
+      <c r="L21" s="119"/>
+      <c r="M21" s="139"/>
+      <c r="O21" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P21" s="123"/>
-      <c r="Q21" s="124" t="s">
+      <c r="P21" s="137"/>
+      <c r="Q21" s="138" t="s">
         <v>160</v>
       </c>
-      <c r="R21" s="125"/>
-      <c r="S21" s="126"/>
+      <c r="R21" s="119"/>
+      <c r="S21" s="139"/>
     </row>
     <row r="22" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="33">
@@ -3829,7 +3893,7 @@
         <v>5</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D22" s="90" t="s">
         <v>20</v>
@@ -3838,30 +3902,30 @@
         <v>78</v>
       </c>
       <c r="F22" s="103" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="127" t="s">
+      <c r="J22" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K22" s="127"/>
-      <c r="L22" s="127"/>
+      <c r="K22" s="128"/>
+      <c r="L22" s="128"/>
       <c r="M22" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="127" t="s">
+      <c r="P22" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q22" s="127"/>
-      <c r="R22" s="127"/>
+      <c r="Q22" s="128"/>
+      <c r="R22" s="128"/>
       <c r="S22" s="69" t="s">
         <v>8</v>
       </c>
@@ -3872,7 +3936,7 @@
         <v>6</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D23" s="1">
         <v>1</v>
@@ -3881,7 +3945,7 @@
         <v>78</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>84</v>
@@ -3889,22 +3953,22 @@
       <c r="I23" s="70">
         <v>1</v>
       </c>
-      <c r="J23" s="136" t="s">
+      <c r="J23" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="136"/>
-      <c r="L23" s="136"/>
+      <c r="K23" s="140"/>
+      <c r="L23" s="140"/>
       <c r="M23" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O23" s="87">
         <v>1</v>
       </c>
-      <c r="P23" s="143" t="s">
+      <c r="P23" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="143"/>
-      <c r="R23" s="143"/>
+      <c r="Q23" s="129"/>
+      <c r="R23" s="129"/>
       <c r="S23" s="88" t="s">
         <v>132</v>
       </c>
@@ -3915,19 +3979,19 @@
         <v>7</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D24" s="1">
         <v>3</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I24" s="67" t="s">
         <v>41</v>
@@ -3947,11 +4011,11 @@
       <c r="O24" s="80">
         <v>2</v>
       </c>
-      <c r="P24" s="125" t="s">
+      <c r="P24" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q24" s="125"/>
-      <c r="R24" s="125"/>
+      <c r="Q24" s="119"/>
+      <c r="R24" s="119"/>
       <c r="S24" s="82" t="s">
         <v>133</v>
       </c>
@@ -3962,7 +4026,7 @@
         <v>8</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D25" s="90" t="s">
         <v>20</v>
@@ -4013,19 +4077,19 @@
         <v>9</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D26" s="1">
         <v>2</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I26" s="76">
         <v>2</v>
@@ -4064,7 +4128,7 @@
         <v>10</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D27" s="90" t="s">
         <v>20</v>
@@ -4076,7 +4140,7 @@
         <v>53</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I27" s="83">
         <v>3</v>
@@ -4115,7 +4179,7 @@
         <v>11</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D28" s="90" t="s">
         <v>21</v>
@@ -4166,19 +4230,19 @@
         <v>12</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D29" s="1">
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I29" s="83">
         <v>5</v>
@@ -4217,16 +4281,16 @@
         <v>13</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D30" s="1">
         <v>1</v>
       </c>
       <c r="E30" s="102" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F30" s="103" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>89</v>
@@ -4268,19 +4332,19 @@
         <v>14</v>
       </c>
       <c r="C31" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D31" s="1">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F31" s="103" t="s">
+        <v>384</v>
+      </c>
+      <c r="G31" s="5" t="s">
         <v>264</v>
-      </c>
-      <c r="D31" s="1">
-        <v>1</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="F31" s="103" t="s">
-        <v>386</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>265</v>
       </c>
       <c r="I31" s="80">
         <v>7</v>
@@ -4319,29 +4383,29 @@
         <v>15</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D32" s="1">
         <v>1</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F32" s="103" t="s">
         <v>63</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="I32" s="137" t="s">
+        <v>310</v>
+      </c>
+      <c r="I32" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J32" s="138"/>
-      <c r="K32" s="139" t="s">
+      <c r="J32" s="124"/>
+      <c r="K32" s="125" t="s">
         <v>78</v>
       </c>
-      <c r="L32" s="140"/>
-      <c r="M32" s="141"/>
+      <c r="L32" s="126"/>
+      <c r="M32" s="127"/>
       <c r="O32" s="83">
         <v>7</v>
       </c>
@@ -4364,19 +4428,19 @@
         <v>16</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D33" s="1">
         <v>6</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="O33" s="83">
         <v>8</v>
@@ -4400,19 +4464,19 @@
         <v>17</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D34" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F34" s="103" t="s">
         <v>63</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="O34" s="83">
         <v>9</v>
@@ -4436,19 +4500,19 @@
         <v>18</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D35" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F35" s="103" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="O35" s="80">
         <v>10</v>
@@ -4472,29 +4536,29 @@
         <v>19</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D36" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F36" s="103" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="O36" s="137" t="s">
+        <v>303</v>
+      </c>
+      <c r="O36" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P36" s="138"/>
-      <c r="Q36" s="139" t="s">
-        <v>237</v>
-      </c>
-      <c r="R36" s="140"/>
-      <c r="S36" s="141"/>
+      <c r="P36" s="124"/>
+      <c r="Q36" s="125" t="s">
+        <v>236</v>
+      </c>
+      <c r="R36" s="126"/>
+      <c r="S36" s="127"/>
     </row>
     <row r="37" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="33">
@@ -4502,19 +4566,19 @@
         <v>20</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D37" s="1">
         <v>1</v>
       </c>
       <c r="E37" s="102" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="F37" s="103" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="38" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -4523,37 +4587,37 @@
         <v>21</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="E38" s="102" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F38" s="103" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="I38" s="119" t="s">
+        <v>361</v>
+      </c>
+      <c r="I38" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J38" s="121"/>
-      <c r="K38" s="119" t="s">
+      <c r="K38" s="120" t="s">
         <v>122</v>
       </c>
-      <c r="L38" s="120"/>
+      <c r="L38" s="122"/>
       <c r="M38" s="121"/>
-      <c r="O38" s="119" t="s">
+      <c r="O38" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P38" s="121"/>
-      <c r="Q38" s="119" t="s">
+      <c r="Q38" s="120" t="s">
         <v>173</v>
       </c>
-      <c r="R38" s="120"/>
+      <c r="R38" s="122"/>
       <c r="S38" s="121"/>
     </row>
     <row r="39" spans="2:19" x14ac:dyDescent="0.3">
@@ -4562,7 +4626,7 @@
         <v>22</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D39" s="90" t="s">
         <v>20</v>
@@ -4576,24 +4640,24 @@
       <c r="G39" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="I39" s="128" t="s">
+      <c r="I39" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J39" s="129"/>
-      <c r="K39" s="130" t="s">
+      <c r="J39" s="131"/>
+      <c r="K39" s="132" t="s">
         <v>123</v>
       </c>
-      <c r="L39" s="131"/>
-      <c r="M39" s="132"/>
-      <c r="O39" s="128" t="s">
+      <c r="L39" s="133"/>
+      <c r="M39" s="134"/>
+      <c r="O39" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P39" s="129"/>
-      <c r="Q39" s="130" t="s">
-        <v>233</v>
-      </c>
-      <c r="R39" s="131"/>
-      <c r="S39" s="132"/>
+      <c r="P39" s="131"/>
+      <c r="Q39" s="132" t="s">
+        <v>232</v>
+      </c>
+      <c r="R39" s="133"/>
+      <c r="S39" s="134"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B40" s="33">
@@ -4601,38 +4665,38 @@
         <v>23</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D40" s="101" t="s">
         <v>20</v>
       </c>
       <c r="E40" s="102" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>36</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="I40" s="128" t="s">
+        <v>230</v>
+      </c>
+      <c r="I40" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J40" s="129"/>
-      <c r="K40" s="130" t="s">
+      <c r="J40" s="131"/>
+      <c r="K40" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="L40" s="131"/>
-      <c r="M40" s="132"/>
-      <c r="O40" s="128" t="s">
+      <c r="L40" s="133"/>
+      <c r="M40" s="134"/>
+      <c r="O40" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P40" s="129"/>
-      <c r="Q40" s="128" t="s">
+      <c r="P40" s="131"/>
+      <c r="Q40" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R40" s="142"/>
-      <c r="S40" s="129"/>
+      <c r="R40" s="135"/>
+      <c r="S40" s="131"/>
     </row>
     <row r="41" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="33">
@@ -4640,7 +4704,7 @@
         <v>24</v>
       </c>
       <c r="C41" s="97" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D41" s="90" t="s">
         <v>21</v>
@@ -4649,29 +4713,29 @@
         <v>36</v>
       </c>
       <c r="F41" s="98" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G41" s="99" t="s">
-        <v>275</v>
-      </c>
-      <c r="I41" s="122" t="s">
+        <v>274</v>
+      </c>
+      <c r="I41" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J41" s="123"/>
-      <c r="K41" s="124" t="s">
+      <c r="J41" s="137"/>
+      <c r="K41" s="138" t="s">
         <v>125</v>
       </c>
-      <c r="L41" s="125"/>
-      <c r="M41" s="126"/>
-      <c r="O41" s="122" t="s">
+      <c r="L41" s="119"/>
+      <c r="M41" s="139"/>
+      <c r="O41" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P41" s="123"/>
-      <c r="Q41" s="124" t="s">
+      <c r="P41" s="137"/>
+      <c r="Q41" s="138" t="s">
         <v>174</v>
       </c>
-      <c r="R41" s="125"/>
-      <c r="S41" s="126"/>
+      <c r="R41" s="119"/>
+      <c r="S41" s="139"/>
     </row>
     <row r="42" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="33">
@@ -4679,7 +4743,7 @@
         <v>25</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D42" s="90" t="s">
         <v>20</v>
@@ -4696,22 +4760,22 @@
       <c r="I42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J42" s="127" t="s">
+      <c r="J42" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K42" s="127"/>
-      <c r="L42" s="127"/>
+      <c r="K42" s="128"/>
+      <c r="L42" s="128"/>
       <c r="M42" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P42" s="127" t="s">
+      <c r="P42" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q42" s="127"/>
-      <c r="R42" s="127"/>
+      <c r="Q42" s="128"/>
+      <c r="R42" s="128"/>
       <c r="S42" s="69" t="s">
         <v>8</v>
       </c>
@@ -4722,39 +4786,39 @@
         <v>26</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D43" s="1">
         <v>1</v>
       </c>
       <c r="E43" s="114" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F43" s="98" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I43" s="70">
         <v>1</v>
       </c>
-      <c r="J43" s="136" t="s">
+      <c r="J43" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="K43" s="136"/>
-      <c r="L43" s="136"/>
+      <c r="K43" s="140"/>
+      <c r="L43" s="140"/>
       <c r="M43" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O43" s="87">
         <v>1</v>
       </c>
-      <c r="P43" s="143" t="s">
+      <c r="P43" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q43" s="143"/>
-      <c r="R43" s="143"/>
+      <c r="Q43" s="129"/>
+      <c r="R43" s="129"/>
       <c r="S43" s="88" t="s">
         <v>132</v>
       </c>
@@ -4765,19 +4829,19 @@
         <v>27</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D44" s="1">
         <v>1</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F44" s="103" t="s">
         <v>237</v>
       </c>
-      <c r="F44" s="103" t="s">
-        <v>238</v>
-      </c>
       <c r="G44" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I44" s="67" t="s">
         <v>41</v>
@@ -4797,11 +4861,11 @@
       <c r="O44" s="80">
         <v>2</v>
       </c>
-      <c r="P44" s="125" t="s">
+      <c r="P44" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="125"/>
-      <c r="R44" s="125"/>
+      <c r="Q44" s="119"/>
+      <c r="R44" s="119"/>
       <c r="S44" s="82" t="s">
         <v>133</v>
       </c>
@@ -4812,19 +4876,19 @@
         <v>28</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D45" s="1">
         <v>1</v>
       </c>
       <c r="E45" s="114" t="s">
+        <v>236</v>
+      </c>
+      <c r="F45" s="114" t="s">
         <v>237</v>
       </c>
-      <c r="F45" s="114" t="s">
-        <v>238</v>
-      </c>
       <c r="G45" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I45" s="72">
         <v>1</v>
@@ -4863,19 +4927,19 @@
         <v>29</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D46" s="90" t="s">
         <v>21</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F46" s="103" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G46" s="99" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I46" s="76">
         <v>2</v>
@@ -4908,25 +4972,25 @@
         <v>154</v>
       </c>
     </row>
-    <row r="47" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="33">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D47" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F47" s="103" t="s">
-        <v>340</v>
+        <v>394</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I47" s="80">
         <v>3</v>
@@ -4965,29 +5029,29 @@
         <v>31</v>
       </c>
       <c r="C48" s="112" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D48" s="113" t="s">
         <v>20</v>
       </c>
       <c r="E48" s="111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F48" s="115" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="G48" s="112" t="s">
-        <v>221</v>
-      </c>
-      <c r="I48" s="137" t="s">
+        <v>220</v>
+      </c>
+      <c r="I48" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J48" s="138"/>
-      <c r="K48" s="139" t="s">
+      <c r="J48" s="124"/>
+      <c r="K48" s="125" t="s">
         <v>65</v>
       </c>
-      <c r="L48" s="140"/>
-      <c r="M48" s="141"/>
+      <c r="L48" s="126"/>
+      <c r="M48" s="127"/>
       <c r="O48" s="83">
         <v>3</v>
       </c>
@@ -5010,7 +5074,7 @@
         <v>32</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D49" s="90" t="s">
         <v>56</v>
@@ -5019,10 +5083,10 @@
         <v>63</v>
       </c>
       <c r="F49" s="103" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="O49" s="83">
         <v>4</v>
@@ -5046,19 +5110,19 @@
         <v>33</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D50" s="1">
         <v>1</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F50" s="103" t="s">
         <v>237</v>
       </c>
-      <c r="F50" s="103" t="s">
-        <v>238</v>
-      </c>
       <c r="G50" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="O50" s="83">
         <v>5</v>
@@ -5082,7 +5146,7 @@
         <v>34</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D51" s="90" t="s">
         <v>49</v>
@@ -5091,19 +5155,19 @@
         <v>47</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="I51" s="119" t="s">
+      <c r="I51" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J51" s="121"/>
-      <c r="K51" s="119" t="s">
+      <c r="K51" s="120" t="s">
         <v>129</v>
       </c>
-      <c r="L51" s="120"/>
+      <c r="L51" s="122"/>
       <c r="M51" s="121"/>
       <c r="O51" s="83">
         <v>6</v>
@@ -5127,13 +5191,13 @@
         <v>35</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D52" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>40</v>
@@ -5141,15 +5205,15 @@
       <c r="G52" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I52" s="128" t="s">
+      <c r="I52" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J52" s="129"/>
-      <c r="K52" s="130" t="s">
+      <c r="J52" s="131"/>
+      <c r="K52" s="132" t="s">
         <v>130</v>
       </c>
-      <c r="L52" s="131"/>
-      <c r="M52" s="132"/>
+      <c r="L52" s="133"/>
+      <c r="M52" s="134"/>
       <c r="O52" s="83">
         <v>7</v>
       </c>
@@ -5172,29 +5236,29 @@
         <v>36</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D53" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F53" s="103" t="s">
         <v>48</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="I53" s="128" t="s">
+        <v>223</v>
+      </c>
+      <c r="I53" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J53" s="129"/>
-      <c r="K53" s="130" t="s">
+      <c r="J53" s="131"/>
+      <c r="K53" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="L53" s="131"/>
-      <c r="M53" s="132"/>
+      <c r="L53" s="133"/>
+      <c r="M53" s="134"/>
       <c r="O53" s="83">
         <v>8</v>
       </c>
@@ -5217,29 +5281,29 @@
         <v>37</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D54" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="I54" s="122" t="s">
+        <v>373</v>
+      </c>
+      <c r="I54" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J54" s="123"/>
-      <c r="K54" s="124" t="s">
+      <c r="J54" s="137"/>
+      <c r="K54" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="L54" s="125"/>
-      <c r="M54" s="126"/>
+      <c r="L54" s="119"/>
+      <c r="M54" s="139"/>
       <c r="O54" s="83">
         <v>9</v>
       </c>
@@ -5262,28 +5326,28 @@
         <v>38</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D55" s="1">
         <v>1</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="I55" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J55" s="127" t="s">
+      <c r="J55" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K55" s="127"/>
-      <c r="L55" s="127"/>
+      <c r="K55" s="128"/>
+      <c r="L55" s="128"/>
       <c r="M55" s="69" t="s">
         <v>8</v>
       </c>
@@ -5309,40 +5373,40 @@
         <v>39</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D56" s="1">
         <v>1</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="I56" s="87">
         <v>1</v>
       </c>
-      <c r="J56" s="143" t="s">
+      <c r="J56" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="143"/>
-      <c r="L56" s="143"/>
+      <c r="K56" s="129"/>
+      <c r="L56" s="129"/>
       <c r="M56" s="88" t="s">
         <v>133</v>
       </c>
-      <c r="O56" s="137" t="s">
+      <c r="O56" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P56" s="138"/>
-      <c r="Q56" s="139" t="s">
-        <v>238</v>
-      </c>
-      <c r="R56" s="140"/>
-      <c r="S56" s="141"/>
+      <c r="P56" s="124"/>
+      <c r="Q56" s="125" t="s">
+        <v>237</v>
+      </c>
+      <c r="R56" s="126"/>
+      <c r="S56" s="127"/>
     </row>
     <row r="57" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="33">
@@ -5350,28 +5414,28 @@
         <v>40</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D57" s="1">
         <v>1</v>
       </c>
       <c r="E57" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F57" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="F57" s="2" t="s">
-        <v>368</v>
-      </c>
       <c r="G57" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I57" s="80">
         <v>2</v>
       </c>
-      <c r="J57" s="125" t="s">
+      <c r="J57" s="119" t="s">
         <v>55</v>
       </c>
-      <c r="K57" s="125"/>
-      <c r="L57" s="125"/>
+      <c r="K57" s="119"/>
+      <c r="L57" s="119"/>
       <c r="M57" s="89" t="s">
         <v>134</v>
       </c>
@@ -5382,19 +5446,19 @@
         <v>41</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D58" s="1">
         <v>1</v>
       </c>
       <c r="E58" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F58" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>368</v>
-      </c>
       <c r="G58" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="I58" s="67" t="s">
         <v>41</v>
@@ -5411,14 +5475,14 @@
       <c r="M58" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="O58" s="119" t="s">
+      <c r="O58" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P58" s="121"/>
-      <c r="Q58" s="119" t="s">
+      <c r="Q58" s="120" t="s">
         <v>184</v>
       </c>
-      <c r="R58" s="120"/>
+      <c r="R58" s="122"/>
       <c r="S58" s="121"/>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.3">
@@ -5427,19 +5491,19 @@
         <v>42</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D59" s="33">
         <v>1</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I59" s="72">
         <v>1</v>
@@ -5456,15 +5520,15 @@
       <c r="M59" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="O59" s="128" t="s">
+      <c r="O59" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P59" s="129"/>
-      <c r="Q59" s="130" t="s">
-        <v>233</v>
-      </c>
-      <c r="R59" s="131"/>
-      <c r="S59" s="132"/>
+      <c r="P59" s="131"/>
+      <c r="Q59" s="132" t="s">
+        <v>232</v>
+      </c>
+      <c r="R59" s="133"/>
+      <c r="S59" s="134"/>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B60" s="33">
@@ -5478,7 +5542,7 @@
         <v>20</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>44</v>
@@ -5501,15 +5565,15 @@
       <c r="M60" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="O60" s="128" t="s">
+      <c r="O60" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P60" s="129"/>
-      <c r="Q60" s="128" t="s">
+      <c r="P60" s="131"/>
+      <c r="Q60" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R60" s="142"/>
-      <c r="S60" s="129"/>
+      <c r="R60" s="135"/>
+      <c r="S60" s="131"/>
     </row>
     <row r="61" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="33">
@@ -5517,7 +5581,7 @@
         <v>44</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D61" s="1">
         <v>3</v>
@@ -5526,10 +5590,10 @@
         <v>58</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I61" s="83">
         <v>3</v>
@@ -5546,15 +5610,15 @@
       <c r="M61" s="85" t="s">
         <v>145</v>
       </c>
-      <c r="O61" s="122" t="s">
+      <c r="O61" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P61" s="123"/>
-      <c r="Q61" s="124" t="s">
+      <c r="P61" s="137"/>
+      <c r="Q61" s="138" t="s">
         <v>185</v>
       </c>
-      <c r="R61" s="125"/>
-      <c r="S61" s="126"/>
+      <c r="R61" s="119"/>
+      <c r="S61" s="139"/>
     </row>
     <row r="62" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="33">
@@ -5562,7 +5626,7 @@
         <v>45</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D62" s="1">
         <v>2</v>
@@ -5571,10 +5635,10 @@
         <v>58</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I62" s="83">
         <v>4</v>
@@ -5594,11 +5658,11 @@
       <c r="O62" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P62" s="127" t="s">
+      <c r="P62" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q62" s="127"/>
-      <c r="R62" s="127"/>
+      <c r="Q62" s="128"/>
+      <c r="R62" s="128"/>
       <c r="S62" s="69" t="s">
         <v>8</v>
       </c>
@@ -5609,7 +5673,7 @@
         <v>46</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D63" s="1">
         <v>1</v>
@@ -5618,10 +5682,10 @@
         <v>58</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I63" s="83">
         <v>5</v>
@@ -5641,11 +5705,11 @@
       <c r="O63" s="87">
         <v>1</v>
       </c>
-      <c r="P63" s="143" t="s">
+      <c r="P63" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q63" s="143"/>
-      <c r="R63" s="143"/>
+      <c r="Q63" s="129"/>
+      <c r="R63" s="129"/>
       <c r="S63" s="88" t="s">
         <v>132</v>
       </c>
@@ -5656,7 +5720,7 @@
         <v>47</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D64" s="90" t="s">
         <v>57</v>
@@ -5688,22 +5752,22 @@
       <c r="O64" s="80">
         <v>2</v>
       </c>
-      <c r="P64" s="125" t="s">
+      <c r="P64" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q64" s="125"/>
-      <c r="R64" s="125"/>
+      <c r="Q64" s="119"/>
+      <c r="R64" s="119"/>
       <c r="S64" s="82" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="65" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="33">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D65" s="1">
         <v>6</v>
@@ -5711,11 +5775,11 @@
       <c r="E65" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F65" s="2" t="s">
-        <v>237</v>
+      <c r="F65" s="103" t="s">
+        <v>393</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I65" s="83">
         <v>7</v>
@@ -5754,7 +5818,7 @@
         <v>49</v>
       </c>
       <c r="C66" s="97" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D66" s="101" t="s">
         <v>45</v>
@@ -5805,7 +5869,7 @@
         <v>50</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D67" s="90" t="s">
         <v>55</v>
@@ -5856,7 +5920,7 @@
         <v>51</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D68" s="90" t="s">
         <v>56</v>
@@ -5865,10 +5929,10 @@
         <v>44</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="I68" s="83">
         <v>10</v>
@@ -5907,7 +5971,7 @@
         <v>52</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D69" s="90" t="s">
         <v>56</v>
@@ -5916,10 +5980,10 @@
         <v>44</v>
       </c>
       <c r="F69" s="103" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="I69" s="83">
         <v>11</v>
@@ -5958,7 +6022,7 @@
         <v>53</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D70" s="90" t="s">
         <v>56</v>
@@ -5967,10 +6031,10 @@
         <v>44</v>
       </c>
       <c r="F70" s="103" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="I70" s="83">
         <v>12</v>
@@ -6009,7 +6073,7 @@
         <v>54</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D71" s="1">
         <v>5</v>
@@ -6060,38 +6124,38 @@
         <v>55</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D72" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="I72" s="137" t="s">
+        <v>215</v>
+      </c>
+      <c r="I72" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J72" s="138"/>
-      <c r="K72" s="139" t="s">
+      <c r="J72" s="124"/>
+      <c r="K72" s="125" t="s">
         <v>58</v>
       </c>
-      <c r="L72" s="140"/>
-      <c r="M72" s="141"/>
-      <c r="O72" s="137" t="s">
+      <c r="L72" s="126"/>
+      <c r="M72" s="127"/>
+      <c r="O72" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P72" s="138"/>
-      <c r="Q72" s="139" t="s">
-        <v>239</v>
-      </c>
-      <c r="R72" s="140"/>
-      <c r="S72" s="141"/>
+      <c r="P72" s="124"/>
+      <c r="Q72" s="125" t="s">
+        <v>238</v>
+      </c>
+      <c r="R72" s="126"/>
+      <c r="S72" s="127"/>
     </row>
     <row r="73" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B73" s="33">
@@ -6099,19 +6163,19 @@
         <v>56</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D73" s="101" t="s">
         <v>20</v>
       </c>
       <c r="E73" s="102" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="74" spans="2:19" x14ac:dyDescent="0.3">
@@ -6120,7 +6184,7 @@
         <v>57</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D74" s="1">
         <v>1</v>
@@ -6129,10 +6193,10 @@
         <v>58</v>
       </c>
       <c r="F74" s="114" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.3">
@@ -6141,7 +6205,7 @@
         <v>58</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D75" s="1">
         <v>1</v>
@@ -6150,10 +6214,10 @@
         <v>58</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.3">
@@ -6162,7 +6226,7 @@
         <v>59</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D76" s="1">
         <v>1</v>
@@ -6171,10 +6235,10 @@
         <v>58</v>
       </c>
       <c r="F76" s="114" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G76" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="77" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -6183,19 +6247,19 @@
         <v>60</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D77" s="90" t="s">
         <v>21</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F77" s="103" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G77" s="99" t="s">
-        <v>194</v>
+        <v>407</v>
       </c>
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.3">
@@ -6204,7 +6268,7 @@
         <v>61</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D78" s="90" t="s">
         <v>20</v>
@@ -6213,10 +6277,10 @@
         <v>62</v>
       </c>
       <c r="F78" s="111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G78" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.3">
@@ -6225,7 +6289,7 @@
         <v>62</v>
       </c>
       <c r="C79" s="112" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D79" s="113" t="s">
         <v>20</v>
@@ -6234,10 +6298,10 @@
         <v>62</v>
       </c>
       <c r="F79" s="111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G79" s="112" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.3">
@@ -6246,7 +6310,7 @@
         <v>63</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D80" s="1">
         <v>1</v>
@@ -6255,10 +6319,10 @@
         <v>58</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G80" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.3">
@@ -6267,7 +6331,7 @@
         <v>64</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D81" s="1">
         <v>1</v>
@@ -6276,10 +6340,10 @@
         <v>58</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="82" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -6288,7 +6352,7 @@
         <v>65</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D82" s="101" t="s">
         <v>46</v>
@@ -6297,7 +6361,7 @@
         <v>42</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G82" s="5" t="s">
         <v>51</v>
@@ -6309,7 +6373,7 @@
         <v>66</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D83" s="1">
         <v>1</v>
@@ -6321,7 +6385,7 @@
         <v>43</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.3">
@@ -6330,7 +6394,7 @@
         <v>67</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D84" s="90" t="s">
         <v>20</v>
@@ -6339,10 +6403,10 @@
         <v>43</v>
       </c>
       <c r="F84" s="103" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G84" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.3">
@@ -6360,7 +6424,7 @@
         <v>39</v>
       </c>
       <c r="F85" s="98" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G85" s="99" t="s">
         <v>191</v>
@@ -6372,7 +6436,7 @@
         <v>69</v>
       </c>
       <c r="C86" s="93" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D86" s="92">
         <v>1</v>
@@ -6393,7 +6457,7 @@
         <v>70</v>
       </c>
       <c r="C87" s="93" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D87" s="94" t="s">
         <v>21</v>
@@ -6402,7 +6466,7 @@
         <v>35</v>
       </c>
       <c r="F87" s="95" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="G87" s="96" t="s">
         <v>37</v>
@@ -6414,19 +6478,19 @@
         <v>71</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D88" s="90" t="s">
         <v>21</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>35</v>
       </c>
       <c r="G88" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="89" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6435,19 +6499,19 @@
         <v>72</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="D89" s="1">
         <v>1</v>
       </c>
       <c r="E89" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="F89" s="103" t="s">
         <v>391</v>
       </c>
-      <c r="F89" s="103" t="s">
-        <v>393</v>
-      </c>
       <c r="G89" s="5" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="90" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -6456,19 +6520,19 @@
         <v>73</v>
       </c>
       <c r="C90" s="104" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D90" s="109" t="s">
         <v>20</v>
       </c>
       <c r="E90" s="105" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F90" s="110" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="G90" s="107" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.3">
@@ -6477,19 +6541,19 @@
         <v>74</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="D91" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E91" s="103" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F91" s="103" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G91" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.3">
@@ -6498,19 +6562,19 @@
         <v>75</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D92" s="1">
         <v>1</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F92" s="103" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G92" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.3">
@@ -6519,19 +6583,19 @@
         <v>76</v>
       </c>
       <c r="C93" s="104" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D93" s="105">
         <v>1</v>
       </c>
       <c r="E93" s="105" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F93" s="106" t="s">
         <v>14</v>
       </c>
       <c r="G93" s="107" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.3">
@@ -6540,19 +6604,19 @@
         <v>77</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D94" s="1">
         <v>1</v>
       </c>
       <c r="E94" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F94" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="F94" s="2" t="s">
-        <v>239</v>
-      </c>
       <c r="G94" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="95" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6561,19 +6625,19 @@
         <v>78</v>
       </c>
       <c r="C95" s="104" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D95" s="105">
         <v>1</v>
       </c>
       <c r="E95" s="105" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F95" s="108" t="s">
         <v>73</v>
       </c>
       <c r="G95" s="107" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.3">
@@ -6582,19 +6646,19 @@
         <v>79</v>
       </c>
       <c r="C96" s="112" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D96" s="113" t="s">
         <v>20</v>
       </c>
       <c r="E96" s="111" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F96" s="118" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G96" s="112" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="97" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6603,19 +6667,19 @@
         <v>80</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D97" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F97" s="103" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="98" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6624,19 +6688,19 @@
         <v>81</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D98" s="1">
         <v>1</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F98" s="103" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="99" spans="2:7" x14ac:dyDescent="0.3">
@@ -6645,19 +6709,19 @@
         <v>82</v>
       </c>
       <c r="C99" s="104" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D99" s="109" t="s">
         <v>20</v>
       </c>
       <c r="E99" s="117" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F99" s="106" t="s">
         <v>17</v>
       </c>
       <c r="G99" s="107" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="100" spans="2:7" x14ac:dyDescent="0.3">
@@ -6666,19 +6730,19 @@
         <v>83</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D100" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="101" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
@@ -6687,19 +6751,19 @@
         <v>84</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D101" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F101" s="103" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.3">
@@ -6708,19 +6772,19 @@
         <v>85</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D102" s="1">
         <v>1</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>80</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.3">
@@ -6729,7 +6793,7 @@
         <v>86</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D103" s="90" t="s">
         <v>20</v>
@@ -6741,7 +6805,7 @@
         <v>62</v>
       </c>
       <c r="G103" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="104" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6750,19 +6814,19 @@
         <v>87</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D104" s="90" t="s">
         <v>56</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F104" s="103" t="s">
-        <v>344</v>
+        <v>400</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="105" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6771,60 +6835,129 @@
         <v>88</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>300</v>
+        <v>405</v>
       </c>
       <c r="D105" s="1">
         <v>1</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F105" s="103" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="G105" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B106" s="33" t="str">
+      <c r="B106" s="33">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F106" s="103"/>
-    </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B107" s="33" t="str">
+        <v>89</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D106" s="1">
+        <v>2</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="107" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B107" s="33">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F107" s="103"/>
+        <v>90</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="D107" s="1">
+        <v>2</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F107" s="103" t="s">
+        <v>406</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>398</v>
+      </c>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B108" s="33" t="str">
+      <c r="B108" s="33">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="E108" s="2"/>
-      <c r="F108" s="103"/>
+        <v>91</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="D108" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F108" s="103" t="s">
+        <v>62</v>
+      </c>
+      <c r="G108" s="5" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B109" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F109" s="103"/>
+      <c r="B109" s="33">
+        <f>IF(C109="","",B108+1)</f>
+        <v>92</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="D109" s="90" t="s">
+        <v>21</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G109" s="5" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="110" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B110" s="33" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="F110" s="103"/>
+      <c r="B110" s="33">
+        <f>IF(C110="","",B109+1)</f>
+        <v>93</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="D110" s="90" t="s">
+        <v>21</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F110" s="103" t="s">
+        <v>80</v>
+      </c>
+      <c r="G110" s="5" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B111" s="33" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(C111="","",B110+1)</f>
         <v/>
       </c>
     </row>
@@ -7009,15 +7142,75 @@
     </sortState>
   </autoFilter>
   <mergeCells count="102">
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="Q38:S38"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="J57:L57"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="I54:J54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="J55:L55"/>
+    <mergeCell ref="J56:L56"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:S16"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:S18"/>
     <mergeCell ref="O72:P72"/>
     <mergeCell ref="Q72:S72"/>
     <mergeCell ref="P8:R8"/>
@@ -7042,75 +7235,15 @@
     <mergeCell ref="O36:P36"/>
     <mergeCell ref="Q36:S36"/>
     <mergeCell ref="O19:P19"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="K72:M72"/>
-    <mergeCell ref="J57:L57"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="O5:P5"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="J55:L55"/>
-    <mergeCell ref="J56:L56"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q38:S38"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="P64:R64"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7132,25 +7265,25 @@
   <sheetData>
     <row r="2" spans="2:8" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="102" t="s">
         <v>318</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="102" t="s">
         <v>319</v>
-      </c>
-      <c r="G2" s="102" t="s">
-        <v>320</v>
-      </c>
-      <c r="H2" s="102" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
IDD Update, jal, jr SIM TEST Complete
</commit_message>
<xml_diff>
--- a/document/IDD.xlsx
+++ b/document/IDD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4AEC23-592B-415F-B0A4-115DBD096B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54974AFD-0562-4AE2-B869-771DCA299A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9885" yWindow="1335" windowWidth="21600" windowHeight="11385" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU" sheetId="1" r:id="rId1"/>
@@ -2695,16 +2695,58 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2722,52 +2764,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3130,31 +3130,31 @@
   <sheetData>
     <row r="1" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="141" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="142"/>
-      <c r="D2" s="142"/>
-      <c r="E2" s="142"/>
-      <c r="F2" s="142"/>
-      <c r="G2" s="143"/>
-      <c r="I2" s="120" t="s">
+      <c r="B2" s="133" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="134"/>
+      <c r="D2" s="134"/>
+      <c r="E2" s="134"/>
+      <c r="F2" s="134"/>
+      <c r="G2" s="135"/>
+      <c r="I2" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J2" s="121"/>
-      <c r="K2" s="120" t="s">
+      <c r="K2" s="119" t="s">
         <v>96</v>
       </c>
-      <c r="L2" s="122"/>
+      <c r="L2" s="120"/>
       <c r="M2" s="121"/>
-      <c r="O2" s="120" t="s">
+      <c r="O2" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P2" s="121"/>
-      <c r="Q2" s="120" t="s">
+      <c r="Q2" s="119" t="s">
         <v>149</v>
       </c>
-      <c r="R2" s="122"/>
+      <c r="R2" s="120"/>
       <c r="S2" s="121"/>
     </row>
     <row r="3" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3176,24 +3176,24 @@
       <c r="G3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="130" t="s">
+      <c r="I3" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="131"/>
-      <c r="K3" s="132" t="s">
+      <c r="J3" s="129"/>
+      <c r="K3" s="130" t="s">
         <v>109</v>
       </c>
-      <c r="L3" s="133"/>
-      <c r="M3" s="134"/>
-      <c r="O3" s="130" t="s">
+      <c r="L3" s="131"/>
+      <c r="M3" s="132"/>
+      <c r="O3" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="131"/>
-      <c r="Q3" s="132" t="s">
+      <c r="P3" s="129"/>
+      <c r="Q3" s="130" t="s">
         <v>232</v>
       </c>
-      <c r="R3" s="133"/>
-      <c r="S3" s="134"/>
+      <c r="R3" s="131"/>
+      <c r="S3" s="132"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B4" s="35">
@@ -3214,24 +3214,24 @@
       <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J4" s="131"/>
-      <c r="K4" s="130" t="s">
+      <c r="J4" s="129"/>
+      <c r="K4" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="135"/>
-      <c r="M4" s="131"/>
-      <c r="O4" s="130" t="s">
+      <c r="L4" s="142"/>
+      <c r="M4" s="129"/>
+      <c r="O4" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="130" t="s">
+      <c r="P4" s="129"/>
+      <c r="Q4" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R4" s="135"/>
-      <c r="S4" s="131"/>
+      <c r="R4" s="142"/>
+      <c r="S4" s="129"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="54">
@@ -3252,24 +3252,24 @@
       <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="136" t="s">
+      <c r="I5" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="137"/>
-      <c r="K5" s="138" t="s">
+      <c r="J5" s="123"/>
+      <c r="K5" s="124" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="119"/>
-      <c r="M5" s="139"/>
-      <c r="O5" s="136" t="s">
+      <c r="L5" s="125"/>
+      <c r="M5" s="126"/>
+      <c r="O5" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="137"/>
-      <c r="Q5" s="138" t="s">
+      <c r="P5" s="123"/>
+      <c r="Q5" s="124" t="s">
         <v>150</v>
       </c>
-      <c r="R5" s="119"/>
-      <c r="S5" s="139"/>
+      <c r="R5" s="125"/>
+      <c r="S5" s="126"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="55">
@@ -3293,22 +3293,22 @@
       <c r="I6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="128" t="s">
+      <c r="J6" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K6" s="128"/>
-      <c r="L6" s="128"/>
+      <c r="K6" s="127"/>
+      <c r="L6" s="127"/>
       <c r="M6" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="128" t="s">
+      <c r="P6" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q6" s="128"/>
-      <c r="R6" s="128"/>
+      <c r="Q6" s="127"/>
+      <c r="R6" s="127"/>
       <c r="S6" s="69" t="s">
         <v>8</v>
       </c>
@@ -3335,22 +3335,22 @@
       <c r="I7" s="70">
         <v>1</v>
       </c>
-      <c r="J7" s="140" t="s">
+      <c r="J7" s="136" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="140"/>
-      <c r="L7" s="140"/>
+      <c r="K7" s="136"/>
+      <c r="L7" s="136"/>
       <c r="M7" s="71" t="s">
         <v>132</v>
       </c>
       <c r="O7" s="87">
         <v>1</v>
       </c>
-      <c r="P7" s="129" t="s">
+      <c r="P7" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="129"/>
-      <c r="R7" s="129"/>
+      <c r="Q7" s="143"/>
+      <c r="R7" s="143"/>
       <c r="S7" s="88" t="s">
         <v>132</v>
       </c>
@@ -3392,11 +3392,11 @@
       <c r="O8" s="80">
         <v>2</v>
       </c>
-      <c r="P8" s="119" t="s">
+      <c r="P8" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="119"/>
-      <c r="R8" s="119"/>
+      <c r="Q8" s="125"/>
+      <c r="R8" s="125"/>
       <c r="S8" s="82" t="s">
         <v>133</v>
       </c>
@@ -3570,15 +3570,15 @@
       <c r="G12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="123" t="s">
+      <c r="I12" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="124"/>
-      <c r="K12" s="125" t="s">
+      <c r="J12" s="138"/>
+      <c r="K12" s="139" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="126"/>
-      <c r="M12" s="127"/>
+      <c r="L12" s="140"/>
+      <c r="M12" s="141"/>
       <c r="O12" s="72">
         <v>3</v>
       </c>
@@ -3701,15 +3701,15 @@
       </c>
     </row>
     <row r="16" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O16" s="123" t="s">
+      <c r="O16" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P16" s="124"/>
-      <c r="Q16" s="125" t="s">
+      <c r="P16" s="138"/>
+      <c r="Q16" s="139" t="s">
         <v>235</v>
       </c>
-      <c r="R16" s="126"/>
-      <c r="S16" s="127"/>
+      <c r="R16" s="140"/>
+      <c r="S16" s="141"/>
     </row>
     <row r="17" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="90" t="s">
@@ -3751,23 +3751,23 @@
       <c r="G18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="I18" s="120" t="s">
+      <c r="I18" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J18" s="121"/>
-      <c r="K18" s="120" t="s">
+      <c r="K18" s="119" t="s">
         <v>103</v>
       </c>
-      <c r="L18" s="122"/>
+      <c r="L18" s="120"/>
       <c r="M18" s="121"/>
-      <c r="O18" s="120" t="s">
+      <c r="O18" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P18" s="121"/>
-      <c r="Q18" s="120" t="s">
+      <c r="Q18" s="119" t="s">
         <v>159</v>
       </c>
-      <c r="R18" s="122"/>
+      <c r="R18" s="120"/>
       <c r="S18" s="121"/>
     </row>
     <row r="19" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -3790,24 +3790,24 @@
       <c r="G19" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="I19" s="130" t="s">
+      <c r="I19" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J19" s="131"/>
-      <c r="K19" s="132" t="s">
+      <c r="J19" s="129"/>
+      <c r="K19" s="130" t="s">
         <v>110</v>
       </c>
-      <c r="L19" s="133"/>
-      <c r="M19" s="134"/>
-      <c r="O19" s="130" t="s">
+      <c r="L19" s="131"/>
+      <c r="M19" s="132"/>
+      <c r="O19" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P19" s="131"/>
-      <c r="Q19" s="132" t="s">
+      <c r="P19" s="129"/>
+      <c r="Q19" s="130" t="s">
         <v>232</v>
       </c>
-      <c r="R19" s="133"/>
-      <c r="S19" s="134"/>
+      <c r="R19" s="131"/>
+      <c r="S19" s="132"/>
     </row>
     <row r="20" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B20" s="33">
@@ -3829,24 +3829,24 @@
       <c r="G20" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="I20" s="130" t="s">
+      <c r="I20" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J20" s="131"/>
-      <c r="K20" s="132" t="s">
+      <c r="J20" s="129"/>
+      <c r="K20" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="L20" s="133"/>
-      <c r="M20" s="134"/>
-      <c r="O20" s="130" t="s">
+      <c r="L20" s="131"/>
+      <c r="M20" s="132"/>
+      <c r="O20" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="130" t="s">
+      <c r="P20" s="129"/>
+      <c r="Q20" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R20" s="135"/>
-      <c r="S20" s="131"/>
+      <c r="R20" s="142"/>
+      <c r="S20" s="129"/>
     </row>
     <row r="21" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="33">
@@ -3868,24 +3868,24 @@
       <c r="G21" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="I21" s="136" t="s">
+      <c r="I21" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J21" s="137"/>
-      <c r="K21" s="138" t="s">
+      <c r="J21" s="123"/>
+      <c r="K21" s="124" t="s">
         <v>124</v>
       </c>
-      <c r="L21" s="119"/>
-      <c r="M21" s="139"/>
-      <c r="O21" s="136" t="s">
+      <c r="L21" s="125"/>
+      <c r="M21" s="126"/>
+      <c r="O21" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P21" s="137"/>
-      <c r="Q21" s="138" t="s">
+      <c r="P21" s="123"/>
+      <c r="Q21" s="124" t="s">
         <v>160</v>
       </c>
-      <c r="R21" s="119"/>
-      <c r="S21" s="139"/>
+      <c r="R21" s="125"/>
+      <c r="S21" s="126"/>
     </row>
     <row r="22" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="33">
@@ -3910,22 +3910,22 @@
       <c r="I22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="128" t="s">
+      <c r="J22" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K22" s="128"/>
-      <c r="L22" s="128"/>
+      <c r="K22" s="127"/>
+      <c r="L22" s="127"/>
       <c r="M22" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="128" t="s">
+      <c r="P22" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q22" s="128"/>
-      <c r="R22" s="128"/>
+      <c r="Q22" s="127"/>
+      <c r="R22" s="127"/>
       <c r="S22" s="69" t="s">
         <v>8</v>
       </c>
@@ -3953,22 +3953,22 @@
       <c r="I23" s="70">
         <v>1</v>
       </c>
-      <c r="J23" s="140" t="s">
+      <c r="J23" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="140"/>
-      <c r="L23" s="140"/>
+      <c r="K23" s="136"/>
+      <c r="L23" s="136"/>
       <c r="M23" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O23" s="87">
         <v>1</v>
       </c>
-      <c r="P23" s="129" t="s">
+      <c r="P23" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="129"/>
-      <c r="R23" s="129"/>
+      <c r="Q23" s="143"/>
+      <c r="R23" s="143"/>
       <c r="S23" s="88" t="s">
         <v>132</v>
       </c>
@@ -4011,11 +4011,11 @@
       <c r="O24" s="80">
         <v>2</v>
       </c>
-      <c r="P24" s="119" t="s">
+      <c r="P24" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q24" s="119"/>
-      <c r="R24" s="119"/>
+      <c r="Q24" s="125"/>
+      <c r="R24" s="125"/>
       <c r="S24" s="82" t="s">
         <v>133</v>
       </c>
@@ -4397,15 +4397,15 @@
       <c r="G32" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="I32" s="123" t="s">
+      <c r="I32" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J32" s="124"/>
-      <c r="K32" s="125" t="s">
+      <c r="J32" s="138"/>
+      <c r="K32" s="139" t="s">
         <v>78</v>
       </c>
-      <c r="L32" s="126"/>
-      <c r="M32" s="127"/>
+      <c r="L32" s="140"/>
+      <c r="M32" s="141"/>
       <c r="O32" s="83">
         <v>7</v>
       </c>
@@ -4550,15 +4550,15 @@
       <c r="G36" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="O36" s="123" t="s">
+      <c r="O36" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P36" s="124"/>
-      <c r="Q36" s="125" t="s">
+      <c r="P36" s="138"/>
+      <c r="Q36" s="139" t="s">
         <v>236</v>
       </c>
-      <c r="R36" s="126"/>
-      <c r="S36" s="127"/>
+      <c r="R36" s="140"/>
+      <c r="S36" s="141"/>
     </row>
     <row r="37" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="33">
@@ -4601,23 +4601,23 @@
       <c r="G38" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="I38" s="120" t="s">
+      <c r="I38" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J38" s="121"/>
-      <c r="K38" s="120" t="s">
+      <c r="K38" s="119" t="s">
         <v>122</v>
       </c>
-      <c r="L38" s="122"/>
+      <c r="L38" s="120"/>
       <c r="M38" s="121"/>
-      <c r="O38" s="120" t="s">
+      <c r="O38" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P38" s="121"/>
-      <c r="Q38" s="120" t="s">
+      <c r="Q38" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="R38" s="122"/>
+      <c r="R38" s="120"/>
       <c r="S38" s="121"/>
     </row>
     <row r="39" spans="2:19" x14ac:dyDescent="0.3">
@@ -4640,24 +4640,24 @@
       <c r="G39" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="I39" s="130" t="s">
+      <c r="I39" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J39" s="131"/>
-      <c r="K39" s="132" t="s">
+      <c r="J39" s="129"/>
+      <c r="K39" s="130" t="s">
         <v>123</v>
       </c>
-      <c r="L39" s="133"/>
-      <c r="M39" s="134"/>
-      <c r="O39" s="130" t="s">
+      <c r="L39" s="131"/>
+      <c r="M39" s="132"/>
+      <c r="O39" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P39" s="131"/>
-      <c r="Q39" s="132" t="s">
+      <c r="P39" s="129"/>
+      <c r="Q39" s="130" t="s">
         <v>232</v>
       </c>
-      <c r="R39" s="133"/>
-      <c r="S39" s="134"/>
+      <c r="R39" s="131"/>
+      <c r="S39" s="132"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B40" s="33">
@@ -4679,24 +4679,24 @@
       <c r="G40" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="I40" s="130" t="s">
+      <c r="I40" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J40" s="131"/>
-      <c r="K40" s="132" t="s">
+      <c r="J40" s="129"/>
+      <c r="K40" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="L40" s="133"/>
-      <c r="M40" s="134"/>
-      <c r="O40" s="130" t="s">
+      <c r="L40" s="131"/>
+      <c r="M40" s="132"/>
+      <c r="O40" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P40" s="131"/>
-      <c r="Q40" s="130" t="s">
+      <c r="P40" s="129"/>
+      <c r="Q40" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R40" s="135"/>
-      <c r="S40" s="131"/>
+      <c r="R40" s="142"/>
+      <c r="S40" s="129"/>
     </row>
     <row r="41" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="33">
@@ -4718,24 +4718,24 @@
       <c r="G41" s="99" t="s">
         <v>274</v>
       </c>
-      <c r="I41" s="136" t="s">
+      <c r="I41" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J41" s="137"/>
-      <c r="K41" s="138" t="s">
+      <c r="J41" s="123"/>
+      <c r="K41" s="124" t="s">
         <v>125</v>
       </c>
-      <c r="L41" s="119"/>
-      <c r="M41" s="139"/>
-      <c r="O41" s="136" t="s">
+      <c r="L41" s="125"/>
+      <c r="M41" s="126"/>
+      <c r="O41" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P41" s="137"/>
-      <c r="Q41" s="138" t="s">
+      <c r="P41" s="123"/>
+      <c r="Q41" s="124" t="s">
         <v>174</v>
       </c>
-      <c r="R41" s="119"/>
-      <c r="S41" s="139"/>
+      <c r="R41" s="125"/>
+      <c r="S41" s="126"/>
     </row>
     <row r="42" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="33">
@@ -4760,22 +4760,22 @@
       <c r="I42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J42" s="128" t="s">
+      <c r="J42" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K42" s="128"/>
-      <c r="L42" s="128"/>
+      <c r="K42" s="127"/>
+      <c r="L42" s="127"/>
       <c r="M42" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P42" s="128" t="s">
+      <c r="P42" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q42" s="128"/>
-      <c r="R42" s="128"/>
+      <c r="Q42" s="127"/>
+      <c r="R42" s="127"/>
       <c r="S42" s="69" t="s">
         <v>8</v>
       </c>
@@ -4803,22 +4803,22 @@
       <c r="I43" s="70">
         <v>1</v>
       </c>
-      <c r="J43" s="140" t="s">
+      <c r="J43" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="K43" s="140"/>
-      <c r="L43" s="140"/>
+      <c r="K43" s="136"/>
+      <c r="L43" s="136"/>
       <c r="M43" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O43" s="87">
         <v>1</v>
       </c>
-      <c r="P43" s="129" t="s">
+      <c r="P43" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q43" s="129"/>
-      <c r="R43" s="129"/>
+      <c r="Q43" s="143"/>
+      <c r="R43" s="143"/>
       <c r="S43" s="88" t="s">
         <v>132</v>
       </c>
@@ -4861,11 +4861,11 @@
       <c r="O44" s="80">
         <v>2</v>
       </c>
-      <c r="P44" s="119" t="s">
+      <c r="P44" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="119"/>
-      <c r="R44" s="119"/>
+      <c r="Q44" s="125"/>
+      <c r="R44" s="125"/>
       <c r="S44" s="82" t="s">
         <v>133</v>
       </c>
@@ -5043,15 +5043,15 @@
       <c r="G48" s="112" t="s">
         <v>220</v>
       </c>
-      <c r="I48" s="123" t="s">
+      <c r="I48" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J48" s="124"/>
-      <c r="K48" s="125" t="s">
+      <c r="J48" s="138"/>
+      <c r="K48" s="139" t="s">
         <v>65</v>
       </c>
-      <c r="L48" s="126"/>
-      <c r="M48" s="127"/>
+      <c r="L48" s="140"/>
+      <c r="M48" s="141"/>
       <c r="O48" s="83">
         <v>3</v>
       </c>
@@ -5160,14 +5160,14 @@
       <c r="G51" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="I51" s="120" t="s">
+      <c r="I51" s="119" t="s">
         <v>102</v>
       </c>
       <c r="J51" s="121"/>
-      <c r="K51" s="120" t="s">
+      <c r="K51" s="119" t="s">
         <v>129</v>
       </c>
-      <c r="L51" s="122"/>
+      <c r="L51" s="120"/>
       <c r="M51" s="121"/>
       <c r="O51" s="83">
         <v>6</v>
@@ -5205,15 +5205,15 @@
       <c r="G52" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I52" s="130" t="s">
+      <c r="I52" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="J52" s="131"/>
-      <c r="K52" s="132" t="s">
+      <c r="J52" s="129"/>
+      <c r="K52" s="130" t="s">
         <v>130</v>
       </c>
-      <c r="L52" s="133"/>
-      <c r="M52" s="134"/>
+      <c r="L52" s="131"/>
+      <c r="M52" s="132"/>
       <c r="O52" s="83">
         <v>7</v>
       </c>
@@ -5250,15 +5250,15 @@
       <c r="G53" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="I53" s="130" t="s">
+      <c r="I53" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="J53" s="131"/>
-      <c r="K53" s="132" t="s">
+      <c r="J53" s="129"/>
+      <c r="K53" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="L53" s="133"/>
-      <c r="M53" s="134"/>
+      <c r="L53" s="131"/>
+      <c r="M53" s="132"/>
       <c r="O53" s="83">
         <v>8</v>
       </c>
@@ -5295,15 +5295,15 @@
       <c r="G54" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="I54" s="136" t="s">
+      <c r="I54" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="J54" s="137"/>
-      <c r="K54" s="138" t="s">
+      <c r="J54" s="123"/>
+      <c r="K54" s="124" t="s">
         <v>131</v>
       </c>
-      <c r="L54" s="119"/>
-      <c r="M54" s="139"/>
+      <c r="L54" s="125"/>
+      <c r="M54" s="126"/>
       <c r="O54" s="83">
         <v>9</v>
       </c>
@@ -5343,11 +5343,11 @@
       <c r="I55" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J55" s="128" t="s">
+      <c r="J55" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="K55" s="128"/>
-      <c r="L55" s="128"/>
+      <c r="K55" s="127"/>
+      <c r="L55" s="127"/>
       <c r="M55" s="69" t="s">
         <v>8</v>
       </c>
@@ -5390,23 +5390,23 @@
       <c r="I56" s="87">
         <v>1</v>
       </c>
-      <c r="J56" s="129" t="s">
+      <c r="J56" s="143" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="129"/>
-      <c r="L56" s="129"/>
+      <c r="K56" s="143"/>
+      <c r="L56" s="143"/>
       <c r="M56" s="88" t="s">
         <v>133</v>
       </c>
-      <c r="O56" s="123" t="s">
+      <c r="O56" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P56" s="124"/>
-      <c r="Q56" s="125" t="s">
+      <c r="P56" s="138"/>
+      <c r="Q56" s="139" t="s">
         <v>237</v>
       </c>
-      <c r="R56" s="126"/>
-      <c r="S56" s="127"/>
+      <c r="R56" s="140"/>
+      <c r="S56" s="141"/>
     </row>
     <row r="57" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="33">
@@ -5431,11 +5431,11 @@
       <c r="I57" s="80">
         <v>2</v>
       </c>
-      <c r="J57" s="119" t="s">
+      <c r="J57" s="125" t="s">
         <v>55</v>
       </c>
-      <c r="K57" s="119"/>
-      <c r="L57" s="119"/>
+      <c r="K57" s="125"/>
+      <c r="L57" s="125"/>
       <c r="M57" s="89" t="s">
         <v>134</v>
       </c>
@@ -5475,14 +5475,14 @@
       <c r="M58" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="O58" s="120" t="s">
+      <c r="O58" s="119" t="s">
         <v>102</v>
       </c>
       <c r="P58" s="121"/>
-      <c r="Q58" s="120" t="s">
+      <c r="Q58" s="119" t="s">
         <v>184</v>
       </c>
-      <c r="R58" s="122"/>
+      <c r="R58" s="120"/>
       <c r="S58" s="121"/>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.3">
@@ -5520,15 +5520,15 @@
       <c r="M59" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="O59" s="130" t="s">
+      <c r="O59" s="128" t="s">
         <v>108</v>
       </c>
-      <c r="P59" s="131"/>
-      <c r="Q59" s="132" t="s">
+      <c r="P59" s="129"/>
+      <c r="Q59" s="130" t="s">
         <v>232</v>
       </c>
-      <c r="R59" s="133"/>
-      <c r="S59" s="134"/>
+      <c r="R59" s="131"/>
+      <c r="S59" s="132"/>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B60" s="33">
@@ -5565,15 +5565,15 @@
       <c r="M60" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="O60" s="130" t="s">
+      <c r="O60" s="128" t="s">
         <v>106</v>
       </c>
-      <c r="P60" s="131"/>
-      <c r="Q60" s="130" t="s">
+      <c r="P60" s="129"/>
+      <c r="Q60" s="128" t="s">
         <v>64</v>
       </c>
-      <c r="R60" s="135"/>
-      <c r="S60" s="131"/>
+      <c r="R60" s="142"/>
+      <c r="S60" s="129"/>
     </row>
     <row r="61" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="33">
@@ -5610,15 +5610,15 @@
       <c r="M61" s="85" t="s">
         <v>145</v>
       </c>
-      <c r="O61" s="136" t="s">
+      <c r="O61" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="P61" s="137"/>
-      <c r="Q61" s="138" t="s">
+      <c r="P61" s="123"/>
+      <c r="Q61" s="124" t="s">
         <v>185</v>
       </c>
-      <c r="R61" s="119"/>
-      <c r="S61" s="139"/>
+      <c r="R61" s="125"/>
+      <c r="S61" s="126"/>
     </row>
     <row r="62" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="33">
@@ -5658,11 +5658,11 @@
       <c r="O62" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P62" s="128" t="s">
+      <c r="P62" s="127" t="s">
         <v>97</v>
       </c>
-      <c r="Q62" s="128"/>
-      <c r="R62" s="128"/>
+      <c r="Q62" s="127"/>
+      <c r="R62" s="127"/>
       <c r="S62" s="69" t="s">
         <v>8</v>
       </c>
@@ -5705,11 +5705,11 @@
       <c r="O63" s="87">
         <v>1</v>
       </c>
-      <c r="P63" s="129" t="s">
+      <c r="P63" s="143" t="s">
         <v>21</v>
       </c>
-      <c r="Q63" s="129"/>
-      <c r="R63" s="129"/>
+      <c r="Q63" s="143"/>
+      <c r="R63" s="143"/>
       <c r="S63" s="88" t="s">
         <v>132</v>
       </c>
@@ -5752,11 +5752,11 @@
       <c r="O64" s="80">
         <v>2</v>
       </c>
-      <c r="P64" s="119" t="s">
+      <c r="P64" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="Q64" s="119"/>
-      <c r="R64" s="119"/>
+      <c r="Q64" s="125"/>
+      <c r="R64" s="125"/>
       <c r="S64" s="82" t="s">
         <v>133</v>
       </c>
@@ -6138,24 +6138,24 @@
       <c r="G72" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="I72" s="123" t="s">
+      <c r="I72" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="J72" s="124"/>
-      <c r="K72" s="125" t="s">
+      <c r="J72" s="138"/>
+      <c r="K72" s="139" t="s">
         <v>58</v>
       </c>
-      <c r="L72" s="126"/>
-      <c r="M72" s="127"/>
-      <c r="O72" s="123" t="s">
+      <c r="L72" s="140"/>
+      <c r="M72" s="141"/>
+      <c r="O72" s="137" t="s">
         <v>104</v>
       </c>
-      <c r="P72" s="124"/>
-      <c r="Q72" s="125" t="s">
+      <c r="P72" s="138"/>
+      <c r="Q72" s="139" t="s">
         <v>238</v>
       </c>
-      <c r="R72" s="126"/>
-      <c r="S72" s="127"/>
+      <c r="R72" s="140"/>
+      <c r="S72" s="141"/>
     </row>
     <row r="73" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B73" s="33">
@@ -6582,20 +6582,20 @@
         <f t="shared" si="2"/>
         <v>76</v>
       </c>
-      <c r="C93" s="104" t="s">
-        <v>249</v>
-      </c>
-      <c r="D93" s="105">
-        <v>1</v>
-      </c>
-      <c r="E93" s="105" t="s">
+      <c r="C93" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D93" s="1">
+        <v>2</v>
+      </c>
+      <c r="E93" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F93" s="106" t="s">
-        <v>14</v>
-      </c>
-      <c r="G93" s="107" t="s">
-        <v>251</v>
+      <c r="F93" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.3">
@@ -6603,167 +6603,167 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="C94" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="D94" s="1">
+      <c r="C94" s="104" t="s">
+        <v>249</v>
+      </c>
+      <c r="D94" s="105">
         <v>1</v>
       </c>
-      <c r="E94" s="2" t="s">
+      <c r="E94" s="105" t="s">
         <v>237</v>
       </c>
-      <c r="F94" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G94" s="5" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="95" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="F94" s="106" t="s">
+        <v>14</v>
+      </c>
+      <c r="G94" s="107" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="95" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B95" s="33">
         <f t="shared" si="2"/>
         <v>78</v>
       </c>
-      <c r="C95" s="104" t="s">
-        <v>250</v>
-      </c>
-      <c r="D95" s="105">
+      <c r="C95" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="D95" s="1">
         <v>1</v>
       </c>
-      <c r="E95" s="105" t="s">
+      <c r="E95" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F95" s="108" t="s">
-        <v>73</v>
-      </c>
-      <c r="G95" s="107" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F95" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G95" s="5" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="96" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B96" s="33">
         <f t="shared" si="2"/>
         <v>79</v>
       </c>
-      <c r="C96" s="112" t="s">
-        <v>259</v>
-      </c>
-      <c r="D96" s="113" t="s">
-        <v>20</v>
-      </c>
-      <c r="E96" s="111" t="s">
+      <c r="C96" s="104" t="s">
+        <v>250</v>
+      </c>
+      <c r="D96" s="105">
+        <v>1</v>
+      </c>
+      <c r="E96" s="105" t="s">
         <v>237</v>
       </c>
-      <c r="F96" s="118" t="s">
-        <v>331</v>
-      </c>
-      <c r="G96" s="112" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="97" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="F96" s="108" t="s">
+        <v>73</v>
+      </c>
+      <c r="G96" s="107" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="97" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B97" s="33">
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>323</v>
+        <v>403</v>
       </c>
       <c r="D97" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E97" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E97" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F97" s="103" t="s">
-        <v>335</v>
+      <c r="F97" s="2" t="s">
+        <v>238</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="98" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="98" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B98" s="33">
         <f t="shared" si="2"/>
         <v>81</v>
       </c>
-      <c r="C98" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="D98" s="1">
-        <v>1</v>
-      </c>
-      <c r="E98" s="2" t="s">
+      <c r="C98" s="112" t="s">
+        <v>259</v>
+      </c>
+      <c r="D98" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E98" s="111" t="s">
         <v>237</v>
       </c>
-      <c r="F98" s="103" t="s">
-        <v>329</v>
-      </c>
-      <c r="G98" s="5" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F98" s="118" t="s">
+        <v>331</v>
+      </c>
+      <c r="G98" s="112" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="99" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B99" s="33">
         <f t="shared" si="2"/>
         <v>82</v>
       </c>
-      <c r="C99" s="104" t="s">
-        <v>351</v>
-      </c>
-      <c r="D99" s="109" t="s">
-        <v>20</v>
-      </c>
-      <c r="E99" s="117" t="s">
-        <v>331</v>
-      </c>
-      <c r="F99" s="106" t="s">
-        <v>17</v>
-      </c>
-      <c r="G99" s="107" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="C99" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D99" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F99" s="103" t="s">
+        <v>335</v>
+      </c>
+      <c r="G99" s="5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="100" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B100" s="33">
         <f t="shared" si="2"/>
         <v>83</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="D100" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E100" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="D100" s="1">
+        <v>1</v>
+      </c>
+      <c r="E100" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F100" s="1" t="s">
-        <v>331</v>
+      <c r="F100" s="103" t="s">
+        <v>329</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="101" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="101" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B101" s="33">
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
-      <c r="C101" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="D101" s="90" t="s">
+      <c r="C101" s="104" t="s">
+        <v>351</v>
+      </c>
+      <c r="D101" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="E101" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F101" s="103" t="s">
-        <v>371</v>
-      </c>
-      <c r="G101" s="5" t="s">
-        <v>272</v>
+      <c r="E101" s="117" t="s">
+        <v>331</v>
+      </c>
+      <c r="F101" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="G101" s="107" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.3">
@@ -6772,40 +6772,40 @@
         <v>85</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="D102" s="1">
-        <v>1</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="F102" s="2" t="s">
-        <v>80</v>
+        <v>363</v>
+      </c>
+      <c r="D102" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>331</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.3">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="103" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B103" s="33">
         <f t="shared" si="2"/>
         <v>86</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>288</v>
+        <v>271</v>
       </c>
       <c r="D103" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F103" s="2" t="s">
-        <v>62</v>
+        <v>238</v>
+      </c>
+      <c r="F103" s="103" t="s">
+        <v>371</v>
       </c>
       <c r="G103" s="5" t="s">
-        <v>289</v>
+        <v>272</v>
       </c>
     </row>
     <row r="104" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6814,19 +6814,19 @@
         <v>87</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="D104" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E104" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="D104" s="1">
+        <v>2</v>
+      </c>
+      <c r="E104" s="2" t="s">
         <v>238</v>
       </c>
       <c r="F104" s="103" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>312</v>
+        <v>398</v>
       </c>
     </row>
     <row r="105" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6856,40 +6856,40 @@
         <v>89</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>395</v>
+        <v>267</v>
       </c>
       <c r="D106" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>238</v>
+        <v>80</v>
       </c>
       <c r="G106" s="5" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="107" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="107" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B107" s="33">
         <f t="shared" si="2"/>
         <v>90</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="D107" s="1">
-        <v>2</v>
-      </c>
-      <c r="E107" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="F107" s="103" t="s">
-        <v>406</v>
+        <v>288</v>
+      </c>
+      <c r="D107" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>62</v>
       </c>
       <c r="G107" s="5" t="s">
-        <v>398</v>
+        <v>289</v>
       </c>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.3">
@@ -6898,19 +6898,19 @@
         <v>91</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="D108" s="90" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>401</v>
+        <v>238</v>
       </c>
       <c r="F108" s="103" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G108" s="5" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.3">
@@ -6919,40 +6919,40 @@
         <v>92</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="D109" s="90" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="F109" s="2" t="s">
-        <v>238</v>
+        <v>401</v>
+      </c>
+      <c r="F109" s="103" t="s">
+        <v>62</v>
       </c>
       <c r="G109" s="5" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.3">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="110" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B110" s="33">
         <f>IF(C110="","",B109+1)</f>
         <v>93</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>404</v>
+        <v>311</v>
       </c>
       <c r="D110" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E110" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E110" s="1" t="s">
         <v>238</v>
       </c>
       <c r="F110" s="103" t="s">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="G110" s="5" t="s">
-        <v>409</v>
+        <v>312</v>
       </c>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.3">
@@ -7142,39 +7142,51 @@
     </sortState>
   </autoFilter>
   <mergeCells count="102">
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q38:S38"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="O72:P72"/>
+    <mergeCell ref="Q72:S72"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="O59:P59"/>
+    <mergeCell ref="Q59:S59"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="Q60:S60"/>
+    <mergeCell ref="O61:P61"/>
+    <mergeCell ref="Q61:S61"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="P43:R43"/>
+    <mergeCell ref="O58:P58"/>
+    <mergeCell ref="Q58:S58"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="Q39:S39"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="Q40:S40"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="Q41:S41"/>
+    <mergeCell ref="P22:R22"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="O36:P36"/>
+    <mergeCell ref="Q36:S36"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:S16"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:S18"/>
     <mergeCell ref="I72:J72"/>
     <mergeCell ref="K72:M72"/>
     <mergeCell ref="J57:L57"/>
@@ -7199,51 +7211,39 @@
     <mergeCell ref="K52:M52"/>
     <mergeCell ref="I40:J40"/>
     <mergeCell ref="K40:M40"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="O72:P72"/>
-    <mergeCell ref="Q72:S72"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="O59:P59"/>
-    <mergeCell ref="Q59:S59"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="Q60:S60"/>
-    <mergeCell ref="O61:P61"/>
-    <mergeCell ref="Q61:S61"/>
-    <mergeCell ref="P42:R42"/>
-    <mergeCell ref="P43:R43"/>
-    <mergeCell ref="O58:P58"/>
-    <mergeCell ref="Q58:S58"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="Q39:S39"/>
-    <mergeCell ref="O40:P40"/>
-    <mergeCell ref="Q40:S40"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="Q41:S41"/>
-    <mergeCell ref="P22:R22"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="O36:P36"/>
-    <mergeCell ref="Q36:S36"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="Q38:S38"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update CPU (Add REGIMM)
</commit_message>
<xml_diff>
--- a/document/IDD.xlsx
+++ b/document/IDD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54974AFD-0562-4AE2-B869-771DCA299A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F2A8C6-3745-48F0-9CAF-2E05DA71981D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{813C5046-60F0-40FF-AAC7-48B46C31F73B}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="정리용" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CPU!$C$17:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CPU!$C$17:$G$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="413">
   <si>
     <t>top_cpu</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1712,6 +1712,21 @@
   </si>
   <si>
     <t>PC ADDR (WB)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_registers
+u_control_unit
+u_id_ex_bridge
+u_load_stall_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>w_ex_alu_negative</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ALU Negative Out</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2695,13 +2710,55 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2713,28 +2770,10 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2744,30 +2783,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3130,31 +3145,31 @@
   <sheetData>
     <row r="1" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="133" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="134"/>
-      <c r="D2" s="134"/>
-      <c r="E2" s="134"/>
-      <c r="F2" s="134"/>
-      <c r="G2" s="135"/>
-      <c r="I2" s="119" t="s">
+      <c r="B2" s="141" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="143"/>
+      <c r="I2" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J2" s="121"/>
-      <c r="K2" s="119" t="s">
+      <c r="K2" s="120" t="s">
         <v>96</v>
       </c>
-      <c r="L2" s="120"/>
+      <c r="L2" s="122"/>
       <c r="M2" s="121"/>
-      <c r="O2" s="119" t="s">
+      <c r="O2" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P2" s="121"/>
-      <c r="Q2" s="119" t="s">
+      <c r="Q2" s="120" t="s">
         <v>149</v>
       </c>
-      <c r="R2" s="120"/>
+      <c r="R2" s="122"/>
       <c r="S2" s="121"/>
     </row>
     <row r="3" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3176,24 +3191,24 @@
       <c r="G3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="128" t="s">
+      <c r="I3" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="129"/>
-      <c r="K3" s="130" t="s">
+      <c r="J3" s="131"/>
+      <c r="K3" s="132" t="s">
         <v>109</v>
       </c>
-      <c r="L3" s="131"/>
-      <c r="M3" s="132"/>
-      <c r="O3" s="128" t="s">
+      <c r="L3" s="133"/>
+      <c r="M3" s="134"/>
+      <c r="O3" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="129"/>
-      <c r="Q3" s="130" t="s">
+      <c r="P3" s="131"/>
+      <c r="Q3" s="132" t="s">
         <v>232</v>
       </c>
-      <c r="R3" s="131"/>
-      <c r="S3" s="132"/>
+      <c r="R3" s="133"/>
+      <c r="S3" s="134"/>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B4" s="35">
@@ -3214,24 +3229,24 @@
       <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="128" t="s">
+      <c r="I4" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J4" s="129"/>
-      <c r="K4" s="128" t="s">
+      <c r="J4" s="131"/>
+      <c r="K4" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="142"/>
-      <c r="M4" s="129"/>
-      <c r="O4" s="128" t="s">
+      <c r="L4" s="135"/>
+      <c r="M4" s="131"/>
+      <c r="O4" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P4" s="129"/>
-      <c r="Q4" s="128" t="s">
+      <c r="P4" s="131"/>
+      <c r="Q4" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R4" s="142"/>
-      <c r="S4" s="129"/>
+      <c r="R4" s="135"/>
+      <c r="S4" s="131"/>
     </row>
     <row r="5" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="54">
@@ -3252,24 +3267,24 @@
       <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="122" t="s">
+      <c r="I5" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="123"/>
-      <c r="K5" s="124" t="s">
+      <c r="J5" s="137"/>
+      <c r="K5" s="138" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="125"/>
-      <c r="M5" s="126"/>
-      <c r="O5" s="122" t="s">
+      <c r="L5" s="119"/>
+      <c r="M5" s="139"/>
+      <c r="O5" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="123"/>
-      <c r="Q5" s="124" t="s">
+      <c r="P5" s="137"/>
+      <c r="Q5" s="138" t="s">
         <v>150</v>
       </c>
-      <c r="R5" s="125"/>
-      <c r="S5" s="126"/>
+      <c r="R5" s="119"/>
+      <c r="S5" s="139"/>
     </row>
     <row r="6" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="55">
@@ -3293,22 +3308,22 @@
       <c r="I6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="127" t="s">
+      <c r="J6" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K6" s="127"/>
-      <c r="L6" s="127"/>
+      <c r="K6" s="128"/>
+      <c r="L6" s="128"/>
       <c r="M6" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="127" t="s">
+      <c r="P6" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q6" s="127"/>
-      <c r="R6" s="127"/>
+      <c r="Q6" s="128"/>
+      <c r="R6" s="128"/>
       <c r="S6" s="69" t="s">
         <v>8</v>
       </c>
@@ -3335,22 +3350,22 @@
       <c r="I7" s="70">
         <v>1</v>
       </c>
-      <c r="J7" s="136" t="s">
+      <c r="J7" s="140" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="136"/>
-      <c r="L7" s="136"/>
+      <c r="K7" s="140"/>
+      <c r="L7" s="140"/>
       <c r="M7" s="71" t="s">
         <v>132</v>
       </c>
       <c r="O7" s="87">
         <v>1</v>
       </c>
-      <c r="P7" s="143" t="s">
+      <c r="P7" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="143"/>
-      <c r="R7" s="143"/>
+      <c r="Q7" s="129"/>
+      <c r="R7" s="129"/>
       <c r="S7" s="88" t="s">
         <v>132</v>
       </c>
@@ -3392,11 +3407,11 @@
       <c r="O8" s="80">
         <v>2</v>
       </c>
-      <c r="P8" s="125" t="s">
+      <c r="P8" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q8" s="125"/>
-      <c r="R8" s="125"/>
+      <c r="Q8" s="119"/>
+      <c r="R8" s="119"/>
       <c r="S8" s="82" t="s">
         <v>133</v>
       </c>
@@ -3570,15 +3585,15 @@
       <c r="G12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="137" t="s">
+      <c r="I12" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="138"/>
-      <c r="K12" s="139" t="s">
+      <c r="J12" s="124"/>
+      <c r="K12" s="125" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="140"/>
-      <c r="M12" s="141"/>
+      <c r="L12" s="126"/>
+      <c r="M12" s="127"/>
       <c r="O12" s="72">
         <v>3</v>
       </c>
@@ -3701,15 +3716,15 @@
       </c>
     </row>
     <row r="16" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="O16" s="137" t="s">
+      <c r="O16" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P16" s="138"/>
-      <c r="Q16" s="139" t="s">
+      <c r="P16" s="124"/>
+      <c r="Q16" s="125" t="s">
         <v>235</v>
       </c>
-      <c r="R16" s="140"/>
-      <c r="S16" s="141"/>
+      <c r="R16" s="126"/>
+      <c r="S16" s="127"/>
     </row>
     <row r="17" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="90" t="s">
@@ -3751,23 +3766,23 @@
       <c r="G18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="I18" s="119" t="s">
+      <c r="I18" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J18" s="121"/>
-      <c r="K18" s="119" t="s">
+      <c r="K18" s="120" t="s">
         <v>103</v>
       </c>
-      <c r="L18" s="120"/>
+      <c r="L18" s="122"/>
       <c r="M18" s="121"/>
-      <c r="O18" s="119" t="s">
+      <c r="O18" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P18" s="121"/>
-      <c r="Q18" s="119" t="s">
+      <c r="Q18" s="120" t="s">
         <v>159</v>
       </c>
-      <c r="R18" s="120"/>
+      <c r="R18" s="122"/>
       <c r="S18" s="121"/>
     </row>
     <row r="19" spans="2:19" ht="33" x14ac:dyDescent="0.3">
@@ -3790,24 +3805,24 @@
       <c r="G19" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="I19" s="128" t="s">
+      <c r="I19" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J19" s="129"/>
-      <c r="K19" s="130" t="s">
+      <c r="J19" s="131"/>
+      <c r="K19" s="132" t="s">
         <v>110</v>
       </c>
-      <c r="L19" s="131"/>
-      <c r="M19" s="132"/>
-      <c r="O19" s="128" t="s">
+      <c r="L19" s="133"/>
+      <c r="M19" s="134"/>
+      <c r="O19" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P19" s="129"/>
-      <c r="Q19" s="130" t="s">
+      <c r="P19" s="131"/>
+      <c r="Q19" s="132" t="s">
         <v>232</v>
       </c>
-      <c r="R19" s="131"/>
-      <c r="S19" s="132"/>
+      <c r="R19" s="133"/>
+      <c r="S19" s="134"/>
     </row>
     <row r="20" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B20" s="33">
@@ -3829,24 +3844,24 @@
       <c r="G20" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="I20" s="128" t="s">
+      <c r="I20" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J20" s="129"/>
-      <c r="K20" s="130" t="s">
+      <c r="J20" s="131"/>
+      <c r="K20" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="L20" s="131"/>
-      <c r="M20" s="132"/>
-      <c r="O20" s="128" t="s">
+      <c r="L20" s="133"/>
+      <c r="M20" s="134"/>
+      <c r="O20" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P20" s="129"/>
-      <c r="Q20" s="128" t="s">
+      <c r="P20" s="131"/>
+      <c r="Q20" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R20" s="142"/>
-      <c r="S20" s="129"/>
+      <c r="R20" s="135"/>
+      <c r="S20" s="131"/>
     </row>
     <row r="21" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="33">
@@ -3868,107 +3883,107 @@
       <c r="G21" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="I21" s="122" t="s">
+      <c r="I21" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J21" s="123"/>
-      <c r="K21" s="124" t="s">
+      <c r="J21" s="137"/>
+      <c r="K21" s="138" t="s">
         <v>124</v>
       </c>
-      <c r="L21" s="125"/>
-      <c r="M21" s="126"/>
-      <c r="O21" s="122" t="s">
+      <c r="L21" s="119"/>
+      <c r="M21" s="139"/>
+      <c r="O21" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P21" s="123"/>
-      <c r="Q21" s="124" t="s">
+      <c r="P21" s="137"/>
+      <c r="Q21" s="138" t="s">
         <v>160</v>
       </c>
-      <c r="R21" s="125"/>
-      <c r="S21" s="126"/>
-    </row>
-    <row r="22" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R21" s="119"/>
+      <c r="S21" s="139"/>
+    </row>
+    <row r="22" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="33">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="D22" s="90" t="s">
-        <v>20</v>
+        <v>411</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F22" s="103" t="s">
-        <v>368</v>
+      <c r="F22" s="2" t="s">
+        <v>297</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>257</v>
+        <v>412</v>
       </c>
       <c r="I22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="127" t="s">
+      <c r="J22" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K22" s="127"/>
-      <c r="L22" s="127"/>
+      <c r="K22" s="128"/>
+      <c r="L22" s="128"/>
       <c r="M22" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O22" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="127" t="s">
+      <c r="P22" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q22" s="127"/>
-      <c r="R22" s="127"/>
+      <c r="Q22" s="128"/>
+      <c r="R22" s="128"/>
       <c r="S22" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="33">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D23" s="1">
-        <v>1</v>
+        <v>256</v>
+      </c>
+      <c r="D23" s="90" t="s">
+        <v>20</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>297</v>
+      <c r="F23" s="103" t="s">
+        <v>368</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>84</v>
+        <v>257</v>
       </c>
       <c r="I23" s="70">
         <v>1</v>
       </c>
-      <c r="J23" s="136" t="s">
+      <c r="J23" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="136"/>
-      <c r="L23" s="136"/>
+      <c r="K23" s="140"/>
+      <c r="L23" s="140"/>
       <c r="M23" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O23" s="87">
         <v>1</v>
       </c>
-      <c r="P23" s="143" t="s">
+      <c r="P23" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="143"/>
-      <c r="R23" s="143"/>
+      <c r="Q23" s="129"/>
+      <c r="R23" s="129"/>
       <c r="S23" s="88" t="s">
         <v>132</v>
       </c>
@@ -3979,19 +3994,19 @@
         <v>7</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>243</v>
+        <v>292</v>
       </c>
       <c r="D24" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>236</v>
+        <v>78</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>65</v>
+        <v>297</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>244</v>
+        <v>84</v>
       </c>
       <c r="I24" s="67" t="s">
         <v>41</v>
@@ -4011,34 +4026,34 @@
       <c r="O24" s="80">
         <v>2</v>
       </c>
-      <c r="P24" s="125" t="s">
+      <c r="P24" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q24" s="125"/>
-      <c r="R24" s="125"/>
+      <c r="Q24" s="119"/>
+      <c r="R24" s="119"/>
       <c r="S24" s="82" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="33">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="D25" s="90" t="s">
-        <v>20</v>
+        <v>243</v>
+      </c>
+      <c r="D25" s="1">
+        <v>4</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F25" s="103" t="s">
-        <v>75</v>
+        <v>236</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>81</v>
+        <v>244</v>
       </c>
       <c r="I25" s="72">
         <v>1</v>
@@ -4071,25 +4086,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B26" s="33">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="D26" s="1">
-        <v>2</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>297</v>
+        <v>290</v>
+      </c>
+      <c r="D26" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" s="103" t="s">
+        <v>75</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>262</v>
+        <v>81</v>
       </c>
       <c r="I26" s="76">
         <v>2</v>
@@ -4128,19 +4143,19 @@
         <v>10</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="D27" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>40</v>
+        <v>261</v>
+      </c>
+      <c r="D27" s="1">
+        <v>3</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>53</v>
+        <v>297</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>231</v>
+        <v>262</v>
       </c>
       <c r="I27" s="83">
         <v>3</v>
@@ -4179,19 +4194,19 @@
         <v>11</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="D28" s="90" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="G28" s="5" t="s">
-        <v>88</v>
+        <v>231</v>
       </c>
       <c r="I28" s="83">
         <v>4</v>
@@ -4230,19 +4245,19 @@
         <v>12</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="D29" s="1">
-        <v>1</v>
+        <v>295</v>
+      </c>
+      <c r="D29" s="90" t="s">
+        <v>21</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>233</v>
+        <v>53</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>226</v>
+        <v>88</v>
       </c>
       <c r="I29" s="83">
         <v>5</v>
@@ -4275,25 +4290,25 @@
         <v>168</v>
       </c>
     </row>
-    <row r="30" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B30" s="33">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>297</v>
+        <v>225</v>
       </c>
       <c r="D30" s="1">
         <v>1</v>
       </c>
-      <c r="E30" s="102" t="s">
-        <v>296</v>
-      </c>
-      <c r="F30" s="103" t="s">
-        <v>383</v>
+      <c r="E30" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>89</v>
+        <v>226</v>
       </c>
       <c r="I30" s="83">
         <v>6</v>
@@ -4332,19 +4347,19 @@
         <v>14</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>263</v>
+        <v>297</v>
       </c>
       <c r="D31" s="1">
-        <v>2</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>236</v>
+        <v>1</v>
+      </c>
+      <c r="E31" s="102" t="s">
+        <v>296</v>
       </c>
       <c r="F31" s="103" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>264</v>
+        <v>89</v>
       </c>
       <c r="I31" s="80">
         <v>7</v>
@@ -4377,35 +4392,35 @@
         <v>169</v>
       </c>
     </row>
-    <row r="32" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="33">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>309</v>
+        <v>263</v>
       </c>
       <c r="D32" s="1">
-        <v>1</v>
-      </c>
-      <c r="E32" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>236</v>
       </c>
       <c r="F32" s="103" t="s">
-        <v>63</v>
+        <v>384</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="I32" s="137" t="s">
+        <v>264</v>
+      </c>
+      <c r="I32" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J32" s="138"/>
-      <c r="K32" s="139" t="s">
+      <c r="J32" s="124"/>
+      <c r="K32" s="125" t="s">
         <v>78</v>
       </c>
-      <c r="L32" s="140"/>
-      <c r="M32" s="141"/>
+      <c r="L32" s="126"/>
+      <c r="M32" s="127"/>
       <c r="O32" s="83">
         <v>7</v>
       </c>
@@ -4428,19 +4443,19 @@
         <v>16</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>241</v>
+        <v>309</v>
       </c>
       <c r="D33" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>65</v>
+        <v>236</v>
+      </c>
+      <c r="F33" s="103" t="s">
+        <v>63</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>242</v>
+        <v>310</v>
       </c>
       <c r="O33" s="83">
         <v>8</v>
@@ -4464,19 +4479,19 @@
         <v>17</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="D34" s="90" t="s">
-        <v>56</v>
+        <v>241</v>
+      </c>
+      <c r="D34" s="1">
+        <v>6</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="F34" s="103" t="s">
-        <v>63</v>
+        <v>233</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>307</v>
+        <v>242</v>
       </c>
       <c r="O34" s="83">
         <v>9</v>
@@ -4500,7 +4515,7 @@
         <v>18</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="D35" s="90" t="s">
         <v>56</v>
@@ -4509,10 +4524,10 @@
         <v>236</v>
       </c>
       <c r="F35" s="103" t="s">
-        <v>341</v>
+        <v>63</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>321</v>
+        <v>307</v>
       </c>
       <c r="O35" s="80">
         <v>10</v>
@@ -4530,13 +4545,13 @@
         <v>172</v>
       </c>
     </row>
-    <row r="36" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="33">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>304</v>
+        <v>320</v>
       </c>
       <c r="D36" s="90" t="s">
         <v>56</v>
@@ -4545,20 +4560,20 @@
         <v>236</v>
       </c>
       <c r="F36" s="103" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="O36" s="137" t="s">
+        <v>321</v>
+      </c>
+      <c r="O36" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P36" s="138"/>
-      <c r="Q36" s="139" t="s">
+      <c r="P36" s="124"/>
+      <c r="Q36" s="125" t="s">
         <v>236</v>
       </c>
-      <c r="R36" s="140"/>
-      <c r="S36" s="141"/>
+      <c r="R36" s="126"/>
+      <c r="S36" s="127"/>
     </row>
     <row r="37" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="33">
@@ -4566,98 +4581,98 @@
         <v>20</v>
       </c>
       <c r="C37" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="D37" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F37" s="103" t="s">
+        <v>336</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="38" spans="2:19" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="B38" s="33">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>385</v>
-      </c>
-      <c r="D37" s="1">
-        <v>1</v>
-      </c>
-      <c r="E37" s="102" t="s">
-        <v>377</v>
-      </c>
-      <c r="F37" s="103" t="s">
-        <v>392</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="38" spans="2:19" ht="33" x14ac:dyDescent="0.3">
-      <c r="B38" s="33">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>343</v>
       </c>
       <c r="D38" s="1">
         <v>1</v>
       </c>
       <c r="E38" s="102" t="s">
+        <v>377</v>
+      </c>
+      <c r="F38" s="103" t="s">
+        <v>392</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="I38" s="120" t="s">
+        <v>102</v>
+      </c>
+      <c r="J38" s="121"/>
+      <c r="K38" s="120" t="s">
+        <v>122</v>
+      </c>
+      <c r="L38" s="122"/>
+      <c r="M38" s="121"/>
+      <c r="O38" s="120" t="s">
+        <v>102</v>
+      </c>
+      <c r="P38" s="121"/>
+      <c r="Q38" s="120" t="s">
+        <v>173</v>
+      </c>
+      <c r="R38" s="122"/>
+      <c r="S38" s="121"/>
+    </row>
+    <row r="39" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+      <c r="B39" s="33">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D39" s="1">
+        <v>1</v>
+      </c>
+      <c r="E39" s="102" t="s">
         <v>344</v>
       </c>
-      <c r="F38" s="103" t="s">
+      <c r="F39" s="103" t="s">
         <v>369</v>
       </c>
-      <c r="G38" s="5" t="s">
+      <c r="G39" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="I38" s="119" t="s">
-        <v>102</v>
-      </c>
-      <c r="J38" s="121"/>
-      <c r="K38" s="119" t="s">
-        <v>122</v>
-      </c>
-      <c r="L38" s="120"/>
-      <c r="M38" s="121"/>
-      <c r="O38" s="119" t="s">
-        <v>102</v>
-      </c>
-      <c r="P38" s="121"/>
-      <c r="Q38" s="119" t="s">
-        <v>173</v>
-      </c>
-      <c r="R38" s="120"/>
-      <c r="S38" s="121"/>
-    </row>
-    <row r="39" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B39" s="33">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D39" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="I39" s="128" t="s">
+      <c r="I39" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J39" s="129"/>
-      <c r="K39" s="130" t="s">
+      <c r="J39" s="131"/>
+      <c r="K39" s="132" t="s">
         <v>123</v>
       </c>
-      <c r="L39" s="131"/>
-      <c r="M39" s="132"/>
-      <c r="O39" s="128" t="s">
+      <c r="L39" s="133"/>
+      <c r="M39" s="134"/>
+      <c r="O39" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P39" s="129"/>
-      <c r="Q39" s="130" t="s">
+      <c r="P39" s="131"/>
+      <c r="Q39" s="132" t="s">
         <v>232</v>
       </c>
-      <c r="R39" s="131"/>
-      <c r="S39" s="132"/>
+      <c r="R39" s="133"/>
+      <c r="S39" s="134"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B40" s="33">
@@ -4665,183 +4680,183 @@
         <v>23</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="D40" s="101" t="s">
+        <v>293</v>
+      </c>
+      <c r="D40" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="E40" s="102" t="s">
-        <v>233</v>
+      <c r="E40" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="I40" s="128" t="s">
+        <v>86</v>
+      </c>
+      <c r="I40" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J40" s="129"/>
-      <c r="K40" s="130" t="s">
+      <c r="J40" s="131"/>
+      <c r="K40" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="L40" s="131"/>
-      <c r="M40" s="132"/>
-      <c r="O40" s="128" t="s">
+      <c r="L40" s="133"/>
+      <c r="M40" s="134"/>
+      <c r="O40" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P40" s="129"/>
-      <c r="Q40" s="128" t="s">
+      <c r="P40" s="131"/>
+      <c r="Q40" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R40" s="142"/>
-      <c r="S40" s="129"/>
+      <c r="R40" s="135"/>
+      <c r="S40" s="131"/>
     </row>
     <row r="41" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="33">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C41" s="97" t="s">
-        <v>273</v>
-      </c>
-      <c r="D41" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E41" s="33" t="s">
+      <c r="C41" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D41" s="101" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" s="102" t="s">
+        <v>233</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F41" s="98" t="s">
-        <v>326</v>
-      </c>
-      <c r="G41" s="99" t="s">
-        <v>274</v>
-      </c>
-      <c r="I41" s="122" t="s">
+      <c r="G41" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="I41" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J41" s="123"/>
-      <c r="K41" s="124" t="s">
+      <c r="J41" s="137"/>
+      <c r="K41" s="138" t="s">
         <v>125</v>
       </c>
-      <c r="L41" s="125"/>
-      <c r="M41" s="126"/>
-      <c r="O41" s="122" t="s">
+      <c r="L41" s="119"/>
+      <c r="M41" s="139"/>
+      <c r="O41" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P41" s="123"/>
-      <c r="Q41" s="124" t="s">
+      <c r="P41" s="137"/>
+      <c r="Q41" s="138" t="s">
         <v>174</v>
       </c>
-      <c r="R41" s="125"/>
-      <c r="S41" s="126"/>
+      <c r="R41" s="119"/>
+      <c r="S41" s="139"/>
     </row>
     <row r="42" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="33">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C42" s="3" t="s">
-        <v>294</v>
+      <c r="C42" s="97" t="s">
+        <v>273</v>
       </c>
       <c r="D42" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>87</v>
+        <v>21</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="F42" s="98" t="s">
+        <v>326</v>
+      </c>
+      <c r="G42" s="99" t="s">
+        <v>274</v>
       </c>
       <c r="I42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J42" s="127" t="s">
+      <c r="J42" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K42" s="127"/>
-      <c r="L42" s="127"/>
+      <c r="K42" s="128"/>
+      <c r="L42" s="128"/>
       <c r="M42" s="69" t="s">
         <v>8</v>
       </c>
       <c r="O42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P42" s="127" t="s">
+      <c r="P42" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q42" s="127"/>
-      <c r="R42" s="127"/>
+      <c r="Q42" s="128"/>
+      <c r="R42" s="128"/>
       <c r="S42" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="33">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1</v>
-      </c>
-      <c r="E43" s="114" t="s">
-        <v>236</v>
-      </c>
-      <c r="F43" s="98" t="s">
-        <v>386</v>
+        <v>294</v>
+      </c>
+      <c r="D43" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>247</v>
+        <v>87</v>
       </c>
       <c r="I43" s="70">
         <v>1</v>
       </c>
-      <c r="J43" s="136" t="s">
+      <c r="J43" s="140" t="s">
         <v>20</v>
       </c>
-      <c r="K43" s="136"/>
-      <c r="L43" s="136"/>
+      <c r="K43" s="140"/>
+      <c r="L43" s="140"/>
       <c r="M43" s="71" t="s">
         <v>133</v>
       </c>
       <c r="O43" s="87">
         <v>1</v>
       </c>
-      <c r="P43" s="143" t="s">
+      <c r="P43" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q43" s="143"/>
-      <c r="R43" s="143"/>
+      <c r="Q43" s="129"/>
+      <c r="R43" s="129"/>
       <c r="S43" s="88" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="44" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="33">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="D44" s="1">
         <v>1</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" s="114" t="s">
         <v>236</v>
       </c>
-      <c r="F44" s="103" t="s">
-        <v>237</v>
+      <c r="F44" s="98" t="s">
+        <v>386</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="I44" s="67" t="s">
         <v>41</v>
@@ -4861,11 +4876,11 @@
       <c r="O44" s="80">
         <v>2</v>
       </c>
-      <c r="P44" s="125" t="s">
+      <c r="P44" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="125"/>
-      <c r="R44" s="125"/>
+      <c r="Q44" s="119"/>
+      <c r="R44" s="119"/>
       <c r="S44" s="82" t="s">
         <v>133</v>
       </c>
@@ -4876,19 +4891,19 @@
         <v>28</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="D45" s="1">
         <v>1</v>
       </c>
-      <c r="E45" s="114" t="s">
+      <c r="E45" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F45" s="114" t="s">
+      <c r="F45" s="103" t="s">
         <v>237</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>248</v>
+        <v>268</v>
       </c>
       <c r="I45" s="72">
         <v>1</v>
@@ -4921,25 +4936,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B46" s="33">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="D46" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="F46" s="103" t="s">
-        <v>254</v>
-      </c>
-      <c r="G46" s="99" t="s">
-        <v>194</v>
+        <v>246</v>
+      </c>
+      <c r="D46" s="1">
+        <v>1</v>
+      </c>
+      <c r="E46" s="114" t="s">
+        <v>236</v>
+      </c>
+      <c r="F46" s="114" t="s">
+        <v>237</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>248</v>
       </c>
       <c r="I46" s="76">
         <v>2</v>
@@ -4978,19 +4993,19 @@
         <v>30</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>217</v>
+        <v>382</v>
       </c>
       <c r="D47" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E47" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>233</v>
       </c>
       <c r="F47" s="103" t="s">
-        <v>394</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>219</v>
+        <v>254</v>
+      </c>
+      <c r="G47" s="99" t="s">
+        <v>194</v>
       </c>
       <c r="I47" s="80">
         <v>3</v>
@@ -5023,35 +5038,35 @@
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="2:19" ht="50.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="33">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C48" s="112" t="s">
-        <v>218</v>
-      </c>
-      <c r="D48" s="113" t="s">
+      <c r="C48" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D48" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="E48" s="111" t="s">
+      <c r="E48" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="F48" s="115" t="s">
-        <v>370</v>
-      </c>
-      <c r="G48" s="112" t="s">
-        <v>220</v>
-      </c>
-      <c r="I48" s="137" t="s">
+      <c r="F48" s="103" t="s">
+        <v>394</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="I48" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="J48" s="138"/>
-      <c r="K48" s="139" t="s">
+      <c r="J48" s="124"/>
+      <c r="K48" s="125" t="s">
         <v>65</v>
       </c>
-      <c r="L48" s="140"/>
-      <c r="M48" s="141"/>
+      <c r="L48" s="126"/>
+      <c r="M48" s="127"/>
       <c r="O48" s="83">
         <v>3</v>
       </c>
@@ -5068,25 +5083,25 @@
         <v>180</v>
       </c>
     </row>
-    <row r="49" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:19" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B49" s="33">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C49" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="D49" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F49" s="103" t="s">
-        <v>386</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>334</v>
+      <c r="C49" s="112" t="s">
+        <v>218</v>
+      </c>
+      <c r="D49" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E49" s="111" t="s">
+        <v>233</v>
+      </c>
+      <c r="F49" s="115" t="s">
+        <v>370</v>
+      </c>
+      <c r="G49" s="112" t="s">
+        <v>220</v>
       </c>
       <c r="O49" s="83">
         <v>4</v>
@@ -5104,25 +5119,25 @@
         <v>181</v>
       </c>
     </row>
-    <row r="50" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="116">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="D50" s="1">
-        <v>1</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>236</v>
+        <v>333</v>
+      </c>
+      <c r="D50" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="F50" s="103" t="s">
-        <v>237</v>
+        <v>386</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>299</v>
+        <v>334</v>
       </c>
       <c r="O50" s="83">
         <v>5</v>
@@ -5146,28 +5161,28 @@
         <v>34</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="D51" s="90" t="s">
-        <v>49</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>279</v>
+        <v>298</v>
+      </c>
+      <c r="D51" s="1">
+        <v>1</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F51" s="103" t="s">
+        <v>237</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="I51" s="119" t="s">
+        <v>299</v>
+      </c>
+      <c r="I51" s="120" t="s">
         <v>102</v>
       </c>
       <c r="J51" s="121"/>
-      <c r="K51" s="119" t="s">
+      <c r="K51" s="120" t="s">
         <v>129</v>
       </c>
-      <c r="L51" s="120"/>
+      <c r="L51" s="122"/>
       <c r="M51" s="121"/>
       <c r="O51" s="83">
         <v>6</v>
@@ -5191,29 +5206,29 @@
         <v>35</v>
       </c>
       <c r="C52" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="D52" s="90" t="s">
+        <v>49</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="D52" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="G52" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I52" s="128" t="s">
+        <v>54</v>
+      </c>
+      <c r="I52" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="J52" s="129"/>
-      <c r="K52" s="130" t="s">
+      <c r="J52" s="131"/>
+      <c r="K52" s="132" t="s">
         <v>130</v>
       </c>
-      <c r="L52" s="131"/>
-      <c r="M52" s="132"/>
+      <c r="L52" s="133"/>
+      <c r="M52" s="134"/>
       <c r="O52" s="83">
         <v>7</v>
       </c>
@@ -5230,35 +5245,35 @@
         <v>182</v>
       </c>
     </row>
-    <row r="53" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B53" s="33">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>221</v>
+        <v>279</v>
       </c>
       <c r="D53" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="F53" s="103" t="s">
-        <v>48</v>
+        <v>278</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="I53" s="128" t="s">
+        <v>52</v>
+      </c>
+      <c r="I53" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="J53" s="129"/>
-      <c r="K53" s="130" t="s">
+      <c r="J53" s="131"/>
+      <c r="K53" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="L53" s="131"/>
-      <c r="M53" s="132"/>
+      <c r="L53" s="133"/>
+      <c r="M53" s="134"/>
       <c r="O53" s="83">
         <v>8</v>
       </c>
@@ -5275,35 +5290,35 @@
         <v>183</v>
       </c>
     </row>
-    <row r="54" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="33">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>372</v>
+        <v>221</v>
       </c>
       <c r="D54" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
+      </c>
+      <c r="F54" s="103" t="s">
+        <v>48</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="I54" s="122" t="s">
+        <v>223</v>
+      </c>
+      <c r="I54" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="J54" s="123"/>
-      <c r="K54" s="124" t="s">
+      <c r="J54" s="137"/>
+      <c r="K54" s="138" t="s">
         <v>131</v>
       </c>
-      <c r="L54" s="125"/>
-      <c r="M54" s="126"/>
+      <c r="L54" s="119"/>
+      <c r="M54" s="139"/>
       <c r="O54" s="83">
         <v>9</v>
       </c>
@@ -5326,28 +5341,28 @@
         <v>38</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="D55" s="1">
-        <v>1</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>365</v>
+        <v>372</v>
+      </c>
+      <c r="D55" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>237</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>356</v>
+        <v>373</v>
       </c>
       <c r="I55" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="J55" s="127" t="s">
+      <c r="J55" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="K55" s="127"/>
-      <c r="L55" s="127"/>
+      <c r="K55" s="128"/>
+      <c r="L55" s="128"/>
       <c r="M55" s="69" t="s">
         <v>8</v>
       </c>
@@ -5373,7 +5388,7 @@
         <v>39</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D56" s="1">
         <v>1</v>
@@ -5385,28 +5400,28 @@
         <v>365</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="I56" s="87">
         <v>1</v>
       </c>
-      <c r="J56" s="143" t="s">
+      <c r="J56" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="K56" s="143"/>
-      <c r="L56" s="143"/>
+      <c r="K56" s="129"/>
+      <c r="L56" s="129"/>
       <c r="M56" s="88" t="s">
         <v>133</v>
       </c>
-      <c r="O56" s="137" t="s">
+      <c r="O56" s="123" t="s">
         <v>104</v>
       </c>
-      <c r="P56" s="138"/>
-      <c r="Q56" s="139" t="s">
+      <c r="P56" s="124"/>
+      <c r="Q56" s="125" t="s">
         <v>237</v>
       </c>
-      <c r="R56" s="140"/>
-      <c r="S56" s="141"/>
+      <c r="R56" s="126"/>
+      <c r="S56" s="127"/>
     </row>
     <row r="57" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B57" s="33">
@@ -5414,7 +5429,7 @@
         <v>40</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D57" s="1">
         <v>1</v>
@@ -5423,19 +5438,19 @@
         <v>364</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I57" s="80">
         <v>2</v>
       </c>
-      <c r="J57" s="125" t="s">
+      <c r="J57" s="119" t="s">
         <v>55</v>
       </c>
-      <c r="K57" s="125"/>
-      <c r="L57" s="125"/>
+      <c r="K57" s="119"/>
+      <c r="L57" s="119"/>
       <c r="M57" s="89" t="s">
         <v>134</v>
       </c>
@@ -5446,7 +5461,7 @@
         <v>41</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D58" s="1">
         <v>1</v>
@@ -5458,7 +5473,7 @@
         <v>366</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I58" s="67" t="s">
         <v>41</v>
@@ -5475,14 +5490,14 @@
       <c r="M58" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="O58" s="119" t="s">
+      <c r="O58" s="120" t="s">
         <v>102</v>
       </c>
       <c r="P58" s="121"/>
-      <c r="Q58" s="119" t="s">
+      <c r="Q58" s="120" t="s">
         <v>184</v>
       </c>
-      <c r="R58" s="120"/>
+      <c r="R58" s="122"/>
       <c r="S58" s="121"/>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.3">
@@ -5491,19 +5506,19 @@
         <v>42</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="D59" s="33">
+        <v>349</v>
+      </c>
+      <c r="D59" s="1">
         <v>1</v>
       </c>
-      <c r="E59" s="1" t="s">
-        <v>344</v>
+      <c r="E59" s="2" t="s">
+        <v>364</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>331</v>
+        <v>366</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I59" s="72">
         <v>1</v>
@@ -5520,15 +5535,15 @@
       <c r="M59" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="O59" s="128" t="s">
+      <c r="O59" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="P59" s="129"/>
-      <c r="Q59" s="130" t="s">
+      <c r="P59" s="131"/>
+      <c r="Q59" s="132" t="s">
         <v>232</v>
       </c>
-      <c r="R59" s="131"/>
-      <c r="S59" s="132"/>
+      <c r="R59" s="133"/>
+      <c r="S59" s="134"/>
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B60" s="33">
@@ -5536,19 +5551,19 @@
         <v>43</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D60" s="90" t="s">
-        <v>20</v>
+        <v>350</v>
+      </c>
+      <c r="D60" s="33">
+        <v>1</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>234</v>
+        <v>344</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>44</v>
+        <v>331</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>193</v>
+        <v>360</v>
       </c>
       <c r="I60" s="76">
         <v>2</v>
@@ -5565,15 +5580,15 @@
       <c r="M60" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="O60" s="128" t="s">
+      <c r="O60" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="P60" s="129"/>
-      <c r="Q60" s="128" t="s">
+      <c r="P60" s="131"/>
+      <c r="Q60" s="130" t="s">
         <v>64</v>
       </c>
-      <c r="R60" s="142"/>
-      <c r="S60" s="129"/>
+      <c r="R60" s="135"/>
+      <c r="S60" s="131"/>
     </row>
     <row r="61" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B61" s="33">
@@ -5581,19 +5596,19 @@
         <v>44</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D61" s="1">
-        <v>3</v>
+        <v>192</v>
+      </c>
+      <c r="D61" s="90" t="s">
+        <v>20</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>58</v>
+        <v>234</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>236</v>
+        <v>44</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="I61" s="83">
         <v>3</v>
@@ -5610,15 +5625,15 @@
       <c r="M61" s="85" t="s">
         <v>145</v>
       </c>
-      <c r="O61" s="122" t="s">
+      <c r="O61" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="P61" s="123"/>
-      <c r="Q61" s="124" t="s">
+      <c r="P61" s="137"/>
+      <c r="Q61" s="138" t="s">
         <v>185</v>
       </c>
-      <c r="R61" s="125"/>
-      <c r="S61" s="126"/>
+      <c r="R61" s="119"/>
+      <c r="S61" s="139"/>
     </row>
     <row r="62" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B62" s="33">
@@ -5626,10 +5641,10 @@
         <v>45</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D62" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>58</v>
@@ -5638,7 +5653,7 @@
         <v>236</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="I62" s="83">
         <v>4</v>
@@ -5658,11 +5673,11 @@
       <c r="O62" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="P62" s="127" t="s">
+      <c r="P62" s="128" t="s">
         <v>97</v>
       </c>
-      <c r="Q62" s="127"/>
-      <c r="R62" s="127"/>
+      <c r="Q62" s="128"/>
+      <c r="R62" s="128"/>
       <c r="S62" s="69" t="s">
         <v>8</v>
       </c>
@@ -5673,19 +5688,19 @@
         <v>46</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D63" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>58</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I63" s="83">
         <v>5</v>
@@ -5705,11 +5720,11 @@
       <c r="O63" s="87">
         <v>1</v>
       </c>
-      <c r="P63" s="143" t="s">
+      <c r="P63" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="Q63" s="143"/>
-      <c r="R63" s="143"/>
+      <c r="Q63" s="129"/>
+      <c r="R63" s="129"/>
       <c r="S63" s="88" t="s">
         <v>132</v>
       </c>
@@ -5720,19 +5735,19 @@
         <v>47</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="D64" s="90" t="s">
-        <v>57</v>
+        <v>196</v>
+      </c>
+      <c r="D64" s="1">
+        <v>1</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>43</v>
+        <v>233</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>61</v>
+        <v>209</v>
       </c>
       <c r="I64" s="83">
         <v>6</v>
@@ -5752,34 +5767,34 @@
       <c r="O64" s="80">
         <v>2</v>
       </c>
-      <c r="P64" s="125" t="s">
+      <c r="P64" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Q64" s="125"/>
-      <c r="R64" s="125"/>
+      <c r="Q64" s="119"/>
+      <c r="R64" s="119"/>
       <c r="S64" s="82" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="65" spans="2:19" ht="33.75" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B65" s="33">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="D65" s="1">
-        <v>6</v>
+        <v>286</v>
+      </c>
+      <c r="D65" s="90" t="s">
+        <v>57</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F65" s="103" t="s">
-        <v>393</v>
+      <c r="F65" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>240</v>
+        <v>61</v>
       </c>
       <c r="I65" s="83">
         <v>7</v>
@@ -5817,20 +5832,20 @@
         <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="C66" s="97" t="s">
-        <v>275</v>
-      </c>
-      <c r="D66" s="101" t="s">
-        <v>45</v>
-      </c>
-      <c r="E66" s="33" t="s">
+      <c r="C66" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D66" s="1">
+        <v>6</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F66" s="98" t="s">
-        <v>42</v>
-      </c>
-      <c r="G66" s="99" t="s">
-        <v>50</v>
+      <c r="F66" s="103" t="s">
+        <v>393</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>240</v>
       </c>
       <c r="I66" s="83">
         <v>8</v>
@@ -5863,25 +5878,25 @@
         <v>154</v>
       </c>
     </row>
-    <row r="67" spans="2:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:19" ht="33" x14ac:dyDescent="0.3">
       <c r="B67" s="33">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="C67" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D67" s="90" t="s">
-        <v>55</v>
-      </c>
-      <c r="E67" s="1" t="s">
+      <c r="C67" s="97" t="s">
+        <v>275</v>
+      </c>
+      <c r="D67" s="101" t="s">
+        <v>45</v>
+      </c>
+      <c r="E67" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="F67" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G67" s="5" t="s">
-        <v>59</v>
+      <c r="F67" s="98" t="s">
+        <v>42</v>
+      </c>
+      <c r="G67" s="99" t="s">
+        <v>50</v>
       </c>
       <c r="I67" s="83">
         <v>9</v>
@@ -5920,19 +5935,19 @@
         <v>51</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D68" s="90" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>236</v>
+        <v>58</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>302</v>
+        <v>59</v>
       </c>
       <c r="I68" s="83">
         <v>10</v>
@@ -5965,13 +5980,13 @@
         <v>28</v>
       </c>
     </row>
-    <row r="69" spans="2:19" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B69" s="33">
         <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D69" s="90" t="s">
         <v>56</v>
@@ -5979,11 +5994,11 @@
       <c r="E69" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F69" s="103" t="s">
-        <v>387</v>
+      <c r="F69" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>322</v>
+        <v>302</v>
       </c>
       <c r="I69" s="83">
         <v>11</v>
@@ -6022,7 +6037,7 @@
         <v>53</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D70" s="90" t="s">
         <v>56</v>
@@ -6034,7 +6049,7 @@
         <v>387</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="I70" s="83">
         <v>12</v>
@@ -6067,25 +6082,25 @@
         <v>188</v>
       </c>
     </row>
-    <row r="71" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:19" ht="66.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B71" s="33">
         <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D71" s="1">
-        <v>5</v>
+        <v>283</v>
+      </c>
+      <c r="D71" s="90" t="s">
+        <v>56</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F71" s="2" t="s">
-        <v>64</v>
+      <c r="F71" s="103" t="s">
+        <v>410</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>60</v>
+        <v>303</v>
       </c>
       <c r="I71" s="80">
         <v>13</v>
@@ -6124,79 +6139,79 @@
         <v>55</v>
       </c>
       <c r="C72" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D72" s="1">
+        <v>5</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I72" s="123" t="s">
+        <v>104</v>
+      </c>
+      <c r="J72" s="124"/>
+      <c r="K72" s="125" t="s">
+        <v>58</v>
+      </c>
+      <c r="L72" s="126"/>
+      <c r="M72" s="127"/>
+      <c r="O72" s="123" t="s">
+        <v>104</v>
+      </c>
+      <c r="P72" s="124"/>
+      <c r="Q72" s="125" t="s">
+        <v>238</v>
+      </c>
+      <c r="R72" s="126"/>
+      <c r="S72" s="127"/>
+    </row>
+    <row r="73" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B73" s="33">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+      <c r="C73" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D73" s="1">
         <v>2</v>
       </c>
-      <c r="E72" s="1" t="s">
+      <c r="E73" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="G72" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="I72" s="137" t="s">
-        <v>104</v>
-      </c>
-      <c r="J72" s="138"/>
-      <c r="K72" s="139" t="s">
-        <v>58</v>
-      </c>
-      <c r="L72" s="140"/>
-      <c r="M72" s="141"/>
-      <c r="O72" s="137" t="s">
-        <v>104</v>
-      </c>
-      <c r="P72" s="138"/>
-      <c r="Q72" s="139" t="s">
-        <v>238</v>
-      </c>
-      <c r="R72" s="140"/>
-      <c r="S72" s="141"/>
-    </row>
-    <row r="73" spans="2:19" ht="33" x14ac:dyDescent="0.3">
-      <c r="B73" s="33">
-        <f t="shared" si="1"/>
-        <v>56</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="D73" s="101" t="s">
-        <v>20</v>
-      </c>
-      <c r="E73" s="102" t="s">
-        <v>380</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>236</v>
       </c>
       <c r="G73" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="74" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+      <c r="B74" s="33">
+        <f t="shared" si="1"/>
+        <v>57</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D74" s="101" t="s">
+        <v>20</v>
+      </c>
+      <c r="E74" s="102" t="s">
+        <v>380</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G74" s="5" t="s">
         <v>228</v>
-      </c>
-    </row>
-    <row r="74" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B74" s="33">
-        <f t="shared" si="1"/>
-        <v>57</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="D74" s="1">
-        <v>1</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F74" s="114" t="s">
-        <v>236</v>
-      </c>
-      <c r="G74" s="5" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.3">
@@ -6205,7 +6220,7 @@
         <v>58</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D75" s="1">
         <v>1</v>
@@ -6213,11 +6228,11 @@
       <c r="E75" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F75" s="2" t="s">
-        <v>233</v>
+      <c r="F75" s="114" t="s">
+        <v>236</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.3">
@@ -6226,7 +6241,7 @@
         <v>59</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D76" s="1">
         <v>1</v>
@@ -6234,53 +6249,53 @@
       <c r="E76" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F76" s="114" t="s">
+      <c r="F76" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="77" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B77" s="33">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="D77" s="1">
+        <v>1</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F77" s="114" t="s">
         <v>236</v>
       </c>
-      <c r="G76" s="5" t="s">
+      <c r="G77" s="5" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="77" spans="2:19" ht="33" x14ac:dyDescent="0.3">
-      <c r="B77" s="33">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="C77" s="3" t="s">
+    <row r="78" spans="2:19" ht="33" x14ac:dyDescent="0.3">
+      <c r="B78" s="33">
+        <f t="shared" si="1"/>
+        <v>61</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="D77" s="90" t="s">
+      <c r="D78" s="90" t="s">
         <v>21</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="E78" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="F77" s="103" t="s">
+      <c r="F78" s="103" t="s">
         <v>253</v>
       </c>
-      <c r="G77" s="99" t="s">
+      <c r="G78" s="99" t="s">
         <v>407</v>
-      </c>
-    </row>
-    <row r="78" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="B78" s="33">
-        <f t="shared" si="1"/>
-        <v>61</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="D78" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F78" s="111" t="s">
-        <v>233</v>
-      </c>
-      <c r="G78" s="5" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.3">
@@ -6288,10 +6303,10 @@
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
-      <c r="C79" s="112" t="s">
-        <v>204</v>
-      </c>
-      <c r="D79" s="113" t="s">
+      <c r="C79" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D79" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E79" s="1" t="s">
@@ -6300,8 +6315,8 @@
       <c r="F79" s="111" t="s">
         <v>233</v>
       </c>
-      <c r="G79" s="112" t="s">
-        <v>206</v>
+      <c r="G79" s="5" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.3">
@@ -6309,20 +6324,20 @@
         <f t="shared" si="1"/>
         <v>63</v>
       </c>
-      <c r="C80" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="D80" s="1">
-        <v>1</v>
+      <c r="C80" s="112" t="s">
+        <v>204</v>
+      </c>
+      <c r="D80" s="113" t="s">
+        <v>20</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="G80" s="5" t="s">
-        <v>208</v>
+        <v>62</v>
+      </c>
+      <c r="F80" s="111" t="s">
+        <v>233</v>
+      </c>
+      <c r="G80" s="112" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.3">
@@ -6331,7 +6346,7 @@
         <v>64</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>198</v>
+        <v>337</v>
       </c>
       <c r="D81" s="1">
         <v>1</v>
@@ -6339,53 +6354,53 @@
       <c r="E81" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="F81" s="1" t="s">
         <v>236</v>
       </c>
       <c r="G81" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B82" s="33">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="D82" s="1">
+        <v>1</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G82" s="5" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
-      <c r="B82" s="33">
-        <f t="shared" si="1"/>
-        <v>65</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="D82" s="101" t="s">
-        <v>46</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="G82" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B83" s="33">
         <f t="shared" ref="B83:B114" si="2">IF(C83="","",B82+1)</f>
         <v>66</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="D83" s="1">
-        <v>1</v>
+        <v>277</v>
+      </c>
+      <c r="D83" s="101" t="s">
+        <v>46</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>43</v>
+        <v>227</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>216</v>
+        <v>51</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.3">
@@ -6394,19 +6409,19 @@
         <v>67</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="D84" s="90" t="s">
-        <v>20</v>
+        <v>202</v>
+      </c>
+      <c r="D84" s="1">
+        <v>1</v>
       </c>
       <c r="E84" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F84" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F84" s="103" t="s">
-        <v>233</v>
-      </c>
       <c r="G84" s="5" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.3">
@@ -6414,20 +6429,20 @@
         <f t="shared" si="2"/>
         <v>68</v>
       </c>
-      <c r="C85" s="97" t="s">
-        <v>190</v>
+      <c r="C85" s="3" t="s">
+        <v>224</v>
       </c>
       <c r="D85" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E85" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="F85" s="98" t="s">
-        <v>326</v>
-      </c>
-      <c r="G85" s="99" t="s">
-        <v>191</v>
+        <v>20</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F85" s="103" t="s">
+        <v>233</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.3">
@@ -6435,125 +6450,125 @@
         <f t="shared" si="2"/>
         <v>69</v>
       </c>
-      <c r="C86" s="93" t="s">
-        <v>276</v>
-      </c>
-      <c r="D86" s="92">
-        <v>1</v>
-      </c>
-      <c r="E86" s="92" t="s">
-        <v>35</v>
-      </c>
-      <c r="F86" s="100" t="s">
-        <v>11</v>
-      </c>
-      <c r="G86" s="96" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="87" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
+      <c r="C86" s="97" t="s">
+        <v>190</v>
+      </c>
+      <c r="D86" s="90" t="s">
+        <v>21</v>
+      </c>
+      <c r="E86" s="33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F86" s="98" t="s">
+        <v>326</v>
+      </c>
+      <c r="G86" s="99" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="87" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B87" s="33">
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
       <c r="C87" s="93" t="s">
-        <v>381</v>
-      </c>
-      <c r="D87" s="94" t="s">
-        <v>21</v>
+        <v>276</v>
+      </c>
+      <c r="D87" s="92">
+        <v>1</v>
       </c>
       <c r="E87" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="F87" s="95" t="s">
-        <v>375</v>
+      <c r="F87" s="100" t="s">
+        <v>11</v>
       </c>
       <c r="G87" s="96" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="88" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B88" s="33">
         <f t="shared" si="2"/>
         <v>71</v>
       </c>
-      <c r="C88" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="D88" s="90" t="s">
+      <c r="C88" s="93" t="s">
+        <v>381</v>
+      </c>
+      <c r="D88" s="94" t="s">
         <v>21</v>
       </c>
-      <c r="E88" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="F88" s="2" t="s">
+      <c r="E88" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="G88" s="5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="89" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="F88" s="95" t="s">
+        <v>375</v>
+      </c>
+      <c r="G88" s="96" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="89" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B89" s="33">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="D89" s="1">
-        <v>1</v>
+        <v>325</v>
+      </c>
+      <c r="D89" s="90" t="s">
+        <v>21</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="F89" s="103" t="s">
-        <v>391</v>
+        <v>326</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="G89" s="5" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="90" spans="2:7" ht="66" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="90" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B90" s="33">
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
-      <c r="C90" s="104" t="s">
-        <v>255</v>
-      </c>
-      <c r="D90" s="109" t="s">
-        <v>20</v>
-      </c>
-      <c r="E90" s="105" t="s">
-        <v>237</v>
-      </c>
-      <c r="F90" s="110" t="s">
-        <v>340</v>
-      </c>
-      <c r="G90" s="107" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="C90" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="D90" s="1">
+        <v>1</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="F90" s="103" t="s">
+        <v>391</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="91" spans="2:7" ht="66" x14ac:dyDescent="0.3">
       <c r="B91" s="33">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
-      <c r="C91" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="D91" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E91" s="103" t="s">
+      <c r="C91" s="104" t="s">
+        <v>255</v>
+      </c>
+      <c r="D91" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="E91" s="105" t="s">
         <v>237</v>
       </c>
-      <c r="F91" s="103" t="s">
-        <v>344</v>
-      </c>
-      <c r="G91" s="5" t="s">
-        <v>308</v>
+      <c r="F91" s="110" t="s">
+        <v>340</v>
+      </c>
+      <c r="G91" s="107" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.3">
@@ -6562,19 +6577,19 @@
         <v>75</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="D92" s="1">
-        <v>1</v>
-      </c>
-      <c r="E92" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D92" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E92" s="103" t="s">
         <v>237</v>
       </c>
       <c r="F92" s="103" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="G92" s="5" t="s">
-        <v>362</v>
+        <v>308</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.3">
@@ -6583,19 +6598,19 @@
         <v>76</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>395</v>
+        <v>345</v>
       </c>
       <c r="D93" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F93" s="2" t="s">
-        <v>238</v>
+      <c r="F93" s="103" t="s">
+        <v>331</v>
       </c>
       <c r="G93" s="5" t="s">
-        <v>397</v>
+        <v>362</v>
       </c>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.3">
@@ -6603,20 +6618,20 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="C94" s="104" t="s">
-        <v>249</v>
-      </c>
-      <c r="D94" s="105">
-        <v>1</v>
-      </c>
-      <c r="E94" s="105" t="s">
+      <c r="C94" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D94" s="1">
+        <v>2</v>
+      </c>
+      <c r="E94" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F94" s="106" t="s">
-        <v>14</v>
-      </c>
-      <c r="G94" s="107" t="s">
-        <v>251</v>
+      <c r="F94" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G94" s="5" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.3">
@@ -6624,62 +6639,62 @@
         <f t="shared" si="2"/>
         <v>78</v>
       </c>
-      <c r="C95" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="D95" s="1">
+      <c r="C95" s="104" t="s">
+        <v>249</v>
+      </c>
+      <c r="D95" s="105">
         <v>1</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E95" s="105" t="s">
         <v>237</v>
       </c>
-      <c r="F95" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G95" s="5" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="96" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="F95" s="106" t="s">
+        <v>14</v>
+      </c>
+      <c r="G95" s="107" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="96" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B96" s="33">
         <f t="shared" si="2"/>
         <v>79</v>
       </c>
-      <c r="C96" s="104" t="s">
-        <v>250</v>
-      </c>
-      <c r="D96" s="105">
+      <c r="C96" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="D96" s="1">
         <v>1</v>
       </c>
-      <c r="E96" s="105" t="s">
+      <c r="E96" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F96" s="108" t="s">
-        <v>73</v>
-      </c>
-      <c r="G96" s="107" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F96" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G96" s="5" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="97" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B97" s="33">
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
-      <c r="C97" s="3" t="s">
-        <v>403</v>
-      </c>
-      <c r="D97" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E97" s="2" t="s">
+      <c r="C97" s="104" t="s">
+        <v>250</v>
+      </c>
+      <c r="D97" s="105">
+        <v>1</v>
+      </c>
+      <c r="E97" s="105" t="s">
         <v>237</v>
       </c>
-      <c r="F97" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G97" s="5" t="s">
-        <v>408</v>
+      <c r="F97" s="108" t="s">
+        <v>73</v>
+      </c>
+      <c r="G97" s="107" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="98" spans="2:7" x14ac:dyDescent="0.3">
@@ -6687,41 +6702,41 @@
         <f t="shared" si="2"/>
         <v>81</v>
       </c>
-      <c r="C98" s="112" t="s">
-        <v>259</v>
-      </c>
-      <c r="D98" s="113" t="s">
-        <v>20</v>
-      </c>
-      <c r="E98" s="111" t="s">
+      <c r="C98" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="D98" s="90" t="s">
+        <v>21</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F98" s="118" t="s">
-        <v>331</v>
-      </c>
-      <c r="G98" s="112" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="99" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="F98" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="99" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B99" s="33">
         <f t="shared" si="2"/>
         <v>82</v>
       </c>
-      <c r="C99" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="D99" s="90" t="s">
-        <v>56</v>
-      </c>
-      <c r="E99" s="1" t="s">
+      <c r="C99" s="112" t="s">
+        <v>259</v>
+      </c>
+      <c r="D99" s="113" t="s">
+        <v>20</v>
+      </c>
+      <c r="E99" s="111" t="s">
         <v>237</v>
       </c>
-      <c r="F99" s="103" t="s">
-        <v>335</v>
-      </c>
-      <c r="G99" s="5" t="s">
-        <v>324</v>
+      <c r="F99" s="118" t="s">
+        <v>331</v>
+      </c>
+      <c r="G99" s="112" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="100" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6730,40 +6745,40 @@
         <v>83</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="D100" s="1">
-        <v>1</v>
-      </c>
-      <c r="E100" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D100" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E100" s="1" t="s">
         <v>237</v>
       </c>
       <c r="F100" s="103" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.3">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="101" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B101" s="33">
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
-      <c r="C101" s="104" t="s">
-        <v>351</v>
-      </c>
-      <c r="D101" s="109" t="s">
-        <v>20</v>
-      </c>
-      <c r="E101" s="117" t="s">
-        <v>331</v>
-      </c>
-      <c r="F101" s="106" t="s">
-        <v>17</v>
-      </c>
-      <c r="G101" s="107" t="s">
-        <v>332</v>
+      <c r="C101" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="D101" s="1">
+        <v>1</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F101" s="103" t="s">
+        <v>329</v>
+      </c>
+      <c r="G101" s="5" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.3">
@@ -6771,62 +6786,62 @@
         <f t="shared" si="2"/>
         <v>85</v>
       </c>
-      <c r="C102" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="D102" s="90" t="s">
+      <c r="C102" s="104" t="s">
+        <v>351</v>
+      </c>
+      <c r="D102" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="E102" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="F102" s="1" t="s">
+      <c r="E102" s="117" t="s">
         <v>331</v>
       </c>
-      <c r="G102" s="5" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="103" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
+      <c r="F102" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="G102" s="107" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="103" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B103" s="33">
         <f t="shared" si="2"/>
         <v>86</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>271</v>
+        <v>363</v>
       </c>
       <c r="D103" s="90" t="s">
         <v>20</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F103" s="103" t="s">
-        <v>371</v>
+        <v>237</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>331</v>
       </c>
       <c r="G103" s="5" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="104" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="104" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
       <c r="B104" s="33">
         <f t="shared" si="2"/>
         <v>87</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="D104" s="1">
-        <v>2</v>
-      </c>
-      <c r="E104" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D104" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="E104" s="1" t="s">
         <v>238</v>
       </c>
       <c r="F104" s="103" t="s">
-        <v>406</v>
+        <v>371</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>398</v>
+        <v>272</v>
       </c>
     </row>
     <row r="105" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -6835,28 +6850,28 @@
         <v>88</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="D105" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>238</v>
       </c>
       <c r="F105" s="103" t="s">
-        <v>342</v>
+        <v>406</v>
       </c>
       <c r="G105" s="5" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.3">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="106" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B106" s="33">
         <f t="shared" si="2"/>
         <v>89</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>267</v>
+        <v>405</v>
       </c>
       <c r="D106" s="1">
         <v>1</v>
@@ -6864,11 +6879,11 @@
       <c r="E106" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="F106" s="2" t="s">
-        <v>80</v>
+      <c r="F106" s="103" t="s">
+        <v>342</v>
       </c>
       <c r="G106" s="5" t="s">
-        <v>270</v>
+        <v>301</v>
       </c>
     </row>
     <row r="107" spans="2:7" x14ac:dyDescent="0.3">
@@ -6877,19 +6892,19 @@
         <v>90</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D107" s="90" t="s">
-        <v>20</v>
-      </c>
-      <c r="E107" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D107" s="1">
+        <v>1</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F107" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F107" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="G107" s="5" t="s">
-        <v>289</v>
+        <v>270</v>
       </c>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.3">
@@ -6898,19 +6913,19 @@
         <v>91</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>404</v>
+        <v>288</v>
       </c>
       <c r="D108" s="90" t="s">
-        <v>21</v>
-      </c>
-      <c r="E108" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="F108" s="103" t="s">
+        <v>20</v>
+      </c>
+      <c r="E108" s="1" t="s">
         <v>80</v>
       </c>
+      <c r="F108" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="G108" s="5" t="s">
-        <v>409</v>
+        <v>289</v>
       </c>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.3">
@@ -6919,46 +6934,61 @@
         <v>92</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="D109" s="90" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>401</v>
+        <v>238</v>
       </c>
       <c r="F109" s="103" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G109" s="5" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="110" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="110" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B110" s="33">
         <f>IF(C110="","",B109+1)</f>
         <v>93</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>311</v>
+        <v>399</v>
       </c>
       <c r="D110" s="90" t="s">
         <v>56</v>
       </c>
-      <c r="E110" s="1" t="s">
+      <c r="E110" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F110" s="103" t="s">
+        <v>62</v>
+      </c>
+      <c r="G110" s="5" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="111" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+      <c r="B111" s="33">
+        <f>IF(C111="","",B110+1)</f>
+        <v>94</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D111" s="90" t="s">
+        <v>56</v>
+      </c>
+      <c r="E111" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="F110" s="103" t="s">
+      <c r="F111" s="103" t="s">
         <v>400</v>
       </c>
-      <c r="G110" s="5" t="s">
+      <c r="G111" s="5" t="s">
         <v>312</v>
-      </c>
-    </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B111" s="33" t="str">
-        <f>IF(C111="","",B110+1)</f>
-        <v/>
       </c>
     </row>
     <row r="112" spans="2:7" x14ac:dyDescent="0.3">
@@ -7136,21 +7166,81 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C17:G17" xr:uid="{4C55C11C-1620-411A-9B2F-3F513CAF246A}">
+  <autoFilter ref="C17:G140" xr:uid="{4C55C11C-1620-411A-9B2F-3F513CAF246A}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C18:G140">
-      <sortCondition ref="C17"/>
+      <sortCondition ref="C17:C140"/>
     </sortState>
   </autoFilter>
   <mergeCells count="102">
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="Q38:S38"/>
-    <mergeCell ref="P44:R44"/>
-    <mergeCell ref="O56:P56"/>
-    <mergeCell ref="Q56:S56"/>
-    <mergeCell ref="P62:R62"/>
-    <mergeCell ref="P63:R63"/>
-    <mergeCell ref="P64:R64"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="J57:L57"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="I54:J54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="J55:L55"/>
+    <mergeCell ref="J56:L56"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:S20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="Q21:S21"/>
+    <mergeCell ref="Q5:S5"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R7"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:S16"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:S18"/>
     <mergeCell ref="O72:P72"/>
     <mergeCell ref="Q72:S72"/>
     <mergeCell ref="P8:R8"/>
@@ -7175,75 +7265,15 @@
     <mergeCell ref="O36:P36"/>
     <mergeCell ref="Q36:S36"/>
     <mergeCell ref="O19:P19"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:S20"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q21:S21"/>
-    <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R7"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:S16"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:S18"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="K72:M72"/>
-    <mergeCell ref="J57:L57"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="O5:P5"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="J55:L55"/>
-    <mergeCell ref="J56:L56"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="J43:L43"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:M19"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q38:S38"/>
+    <mergeCell ref="P44:R44"/>
+    <mergeCell ref="O56:P56"/>
+    <mergeCell ref="Q56:S56"/>
+    <mergeCell ref="P62:R62"/>
+    <mergeCell ref="P63:R63"/>
+    <mergeCell ref="P64:R64"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>